<commit_message>
feat: one-line items with shortened originals
one-line items with shortened originals, decoded item effects, meals

- Items: 391 state what they do in one line. Where original + (data) did
not fit, the sentence was shortened by hand (65, shortened_text.py).
Item effect types decoded with the DT2-2 wiki item list; 55 items left.
- Skills: line 1 that did not fit is shortened (7) or carries its
figures inside the sentence (16). Spiral Arrow and Holy Gavel graded by
their "Damage xn", which the wiki lists as the ATK multiplier. - Meals
(FoodMenuData): stored amounts in place of vague ones; writer exact.

98 tests.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_item_text.xlsx
+++ b/mod_project/data_tables/qol_item_text.xlsx
@@ -769,7 +769,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bread stuffed with yakisoba noodles. Sells out very quickly.</t>
+          <t>Yakisoba noodle bread. Sells out very quickly. (HP/TP +20, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -786,7 +786,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>no room for (HP/TP +20, cures 1 ailment): 89 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Premium steak sandwich with luxury sauce. Extra deluxe.</t>
+          <t>Premium steak sandwich, luxury sauce. Extra deluxe. (HP/TP +30, cures all ailments)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -825,7 +825,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>no room for (HP/TP +30, cures all ailments): 87 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Super spicy curry that would make even a Maharaja groan.</t>
+          <t>Spicy curry that would make even a Maharaja groan. (HP/TP +150, cures all ailments)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -864,7 +864,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>no room for (HP/TP +150, cures all ailments): 89 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Legendary food that's said to make any who eats it fall in love.</t>
+          <t>Legendary food. Whoever eats it falls in love. (HP/TP +1000, cures all ailments)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -903,7 +903,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>no room for (HP/TP +1000, cures all ailments): 98 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>High in nutritional value, it heals HP and TP but is extremely bitter.</t>
+          <t>Highly nutritious, it heals HP and TP but is extremely bitter. (HP +50, TP +20)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>no room for (HP +50, TP +20): 87 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Beard's special bento. A well-balanced meal, and big enough to share.</t>
+          <t>Beard's special bento. Balanced, big enough to share. (party HP +75, party TP +25)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>no room for (party HP +75, party TP +25): 98 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Peggy's eggy milk pudding. It's said to be legendary. (TP +30, sleep 20%)</t>
+          <t>Peggy's eggy milk pudding. It's said to be legendary. (TP +30, 20% sleep)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Kumaya Mangetsudo's anpan. It's low-calorie, but still delicious.</t>
+          <t>Kumaya Mangetsudo's anpan. Low-calorie, but still delicious. (HP/TP +20, 15% sleep)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>no room for (HP/TP +20, sleep 15%): 88 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Mrs. Mary's snack smothered in maple butter. (HP/TP +20, sleep 15%)</t>
+          <t>Mrs. Mary's snack smothered in maple butter. (HP/TP +20, 15% sleep)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Honey-filled monaka sold at the Kumana Mangetsudo. (TP +30, sleep 20%)</t>
+          <t>Honey-filled monaka sold at the Kumana Mangetsudo. (TP +30, 20% sleep)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Consists of Mary Florina's super rich milk collagen. Sorts ailments right out.</t>
+          <t>Mary Florina's rich milk collagen gel. (cures all ailments, restores stats)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>no room for (cures all ailments, restores stats): 115 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>There's a cure for pretty much anything, and there's plenty of it.</t>
+          <t>A cure for anything, and plenty of it. (cures all ailments, restores stats)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>no room for (cures all ailments, restores stats): 103 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>It scrambles your brain, and then you die. No coming back from that.</t>
+          <t>It scrambles your brain, and then you die. No coming back from that. (10% instakill)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -2067,11 +2067,7 @@
           <t>It scrambles your brain, and then you die. No coming back from that (25% Death).</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2091,7 +2087,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Inscribed with impressive wish-granting runes.</t>
+          <t>Inscribed with impressive wish-granting runes. (80% Divine Shield, 80% Insurance)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -2105,11 +2101,7 @@
           <t>Inscribed with impressive wish-granting runes.</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2163,7 +2155,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Rock-hard cracker. Not just a snack, but also an emergency ration!</t>
+          <t>Rock-hard cracker. Snack and emergency ration! (HP/TP +75, cancels Shadow Sew)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2180,7 +2172,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>no room for (HP/TP +75, cancels Shadow Sew): 98 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2304,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>A miraculous wind that once brought spring to the underworld.</t>
+          <t>Wind that brought spring to the underworld. (80% party ATK up, 80% party DEF up)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2328,7 +2320,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2380,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>For those elegant afternoons.</t>
+          <t>For those elegant afternoons. (60% evasion up)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2402,11 +2394,7 @@
           <t>For those elegant afternoons (+60% EVA).</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2426,7 +2414,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Everyone has been looking, and we've finally found it!</t>
+          <t>Everyone has been looking, and we've finally found it! (20% Berserk)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2440,11 +2428,7 @@
           <t>Everyone has been looking, and we've finally found it! (+20% ATK).</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2600,7 +2584,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>When I peeked in, something peeked back... There's someone in there!</t>
+          <t>When I peeked in, something peeked back... There's someone in there! (6% instakill)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2614,11 +2598,7 @@
           <t>When I peeked in, something peeked back... There's someone in there! (25% Death).</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2880,7 +2860,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Whatever's under all that breading, you can bet it's good and fried.</t>
+          <t>Whatever's under the breading, it's good and fried. (HP/TP +175, 75% Berserk)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -2896,7 +2876,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2932,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Those memories are precious... and painful.</t>
+          <t>Those memories are precious... and painful. (20% silence)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -2966,11 +2946,7 @@
           <t>Those memories are precious... and painful (40% Silence).</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3232,7 +3208,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>I must immediately depart on a long, long journey. Don't look for me.</t>
+          <t>I must immediately depart on a long, long journey. Don't look for me. (25% silence)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -3246,11 +3222,7 @@
           <t>I must immediately depart on a long, long journey. Don't look for me (50% Silence).</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3308,7 +3280,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>A red feather you receive after donating to a fundraiser.</t>
+          <t>A red feather you receive after donating to a fundraiser. (TP +150, 75% Berserk)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -3322,11 +3294,7 @@
           <t>A red feather you receive after donating to a fundraiser (+75% ATK).</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3346,7 +3314,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Creepy pitch-black rosary.</t>
+          <t>Creepy pitch-black rosary. (25% stun)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -3360,11 +3328,7 @@
           <t>Creepy pitch-black rosary (50% Blind).</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3384,7 +3348,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Cursed words from an ex-girlfriend. She's really vile...</t>
+          <t>Cursed words from an ex-girlfriend. She's really vile... (30% petrify)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -3399,11 +3363,7 @@
 (Inflict Gray Curse (75% chance).)</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3491,7 +3451,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>One prick with this needle would be disastrous. Handle with care.</t>
+          <t>One prick with this needle would be disastrous. Handle with care. (20% poison)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -3505,11 +3465,7 @@
           <t>One prick with this needle would be disastrous. Handle with care (40% Poison).</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3529,7 +3485,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>A mirror that reveals the truth... You might not want to look.</t>
+          <t>A mirror that reveals the truth... You might not want to look. (15% stun)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -3543,11 +3499,7 @@
           <t>A mirror that reveals the truth... You might not want to look (30% Blind).</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3673,7 +3625,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>You can be a magical girl too.</t>
+          <t>You can be a magical girl too. (40% 2 clones)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -3687,11 +3639,7 @@
           <t>You can be a magical girl too.</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3817,7 +3765,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>A disconcerting egg. The face is always screaming.</t>
+          <t>A disconcerting egg. The face is always screaming. (25% instakill)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -3831,11 +3779,7 @@
           <t>A disconcerting egg. The face is always screaming (90% Death).</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3855,7 +3799,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Clay used for handicraft in the heavens. Heh. They soil themselves.</t>
+          <t>Clay used for handicraft in the heavens. Heh. They soil themselves. (10% 2 clones)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3869,11 +3813,7 @@
           <t>Clay used for handicraft in the heavens. Heh. They soil themselves.</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3893,7 +3833,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Vial of mysterious holy water. Tiny waves are ever-present at the top.</t>
+          <t>Vial of mysterious holy water. Tiny waves ripple at the top. (cures 1 ailment)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -3910,7 +3850,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>no room for (cures 1 ailment): 88 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3872,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Fried up in an iron pan. A steal at 3 million lira!</t>
+          <t>Fried up in an iron pan. A steal at 3 million lira! (HP +50, 20% ATK up)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -3946,11 +3886,7 @@
           <t>Fried up in an iron pan. A steal at 3 million lira! (+20% ATK).</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3970,7 +3906,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>There's no wind blowing, yet you can hear its sound. It cries Mary.</t>
+          <t>There's no wind blowing, yet you can hear its sound. It cries Mary. (15% silence)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -3984,11 +3920,7 @@
           <t>There's no wind blowing, yet you can hear its sound. It cries Mary (30% Silence).</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4080,7 +4012,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Just one drop will refresh constantly overworked eyes.</t>
+          <t>Just one drop will refresh constantly overworked eyes. (80% accuracy up)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4094,11 +4026,7 @@
           <t>Just one drop will refresh constantly overworked eyes (Accuracy +80%.).</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4225,7 +4153,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Make a man out of this and it comes to life. Weird.</t>
+          <t>Make a man out of this and it comes to life. Weird. (30% Insurance)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -4239,11 +4167,7 @@
           <t>Make a man out of this and it comes to life. Weird.</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4297,7 +4221,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>If this is waiting back at the base, you know someone's about to die.</t>
+          <t>If this waits back at base, someone's about to die. (TP +40, 30% instakill)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -4313,7 +4237,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4361,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Moist with the power of life.</t>
+          <t>Moist with the power of life. (50% max HP up)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
@@ -4451,11 +4375,7 @@
           <t>Moist with the power of life.</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4683,7 +4603,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Plan the perfect trip to the world beyond the veil.</t>
+          <t>Plan the perfect trip to the world beyond the veil. (10% instakill)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4697,11 +4617,7 @@
           <t>Plan the perfect trip to the world beyond the veil (20% Death).</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4827,7 +4743,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Smooth, sticky lotion for professional use.</t>
+          <t>Smooth, sticky lotion for professional use. (30% evasion up)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr"/>
@@ -4841,11 +4757,7 @@
           <t>Smooth, sticky lotion for professional use (+30% EVA).</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4899,7 +4811,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>A skull ascended through a secret rite. It's said to grant wishes.</t>
+          <t>A skull from a secret rite. Grants wishes. (60% party ATK up, 30% party magic DEF up)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4915,7 +4827,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -5005,7 +4917,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>A branch only certain people are allowed to pray to. It's twig-sclusive.</t>
+          <t>A branch only some may pray to. It's twig-sclusive. (cures all ailments)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5022,7 +4934,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>no room for (cures all ailments): 93 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -5044,7 +4956,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>A bud of a tree that grows where God resides.</t>
+          <t>A bud of a tree that grows where God resides. (50% party cure-all)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5058,11 +4970,7 @@
           <t>A bud of a tree that grows where God resides.</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5082,7 +4990,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Sandals that are no longer of any use. Might as well toss 'em.</t>
+          <t>Sandals that are no longer of any use. Might as well toss 'em. (15% evasion up)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5096,11 +5004,7 @@
           <t>Sandals that are no longer of any use. Might as well toss 'em (+15% EVA).</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5230,7 +5134,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Stone core made when an evil heart has hardened completely.</t>
+          <t>Stone core made when an evil heart has hardened completely. (20% stun)</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5244,11 +5148,7 @@
           <t>Stone core made when an evil heart has hardened completely (35% Blind).</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5268,7 +5168,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Do YOU ever ruin your good cleaver on bone? Finally, there's help!</t>
+          <t>Do YOU ever ruin your good cleaver on bone? Finally, there's help! (50% ATK up)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5282,11 +5182,7 @@
           <t>Do YOU ever ruin your good cleaver on bone? Finally, there's help! (+50% ATK).</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5451,7 +5347,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>It might be able to take... one more hit. Hit it baby one more time.</t>
+          <t>It might take... one more hit. Hit it baby one more time. (30 fixed damage)</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5467,7 +5363,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5385,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Do the goggles switch her personality, or just give her confidence...?</t>
+          <t>Do the goggles switch her personality, or just add confidence...? (50% max HP up)</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5505,7 +5401,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5495,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Drop made out of collected mirage.</t>
+          <t>Drop made out of collected mirage. (20% Divine Shield)</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5613,11 +5509,7 @@
           <t>Drop made out of collected mirage.</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5637,7 +5529,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>A large, mysterious key made in Hyperborea.</t>
+          <t>A large, mysterious key made in Hyperborea. (40% 1 clone)</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5651,11 +5543,7 @@
           <t>A large, mysterious key made in Hyperborea.</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5675,7 +5563,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Eat this and you may die on the spot... or not at all.</t>
+          <t>Eat this and you may die on the spot... or not at all. (90% instakill, TP +999)</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5689,11 +5577,7 @@
           <t>Eat this and you may die on the spot... or not at all (+999 TP).</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5781,7 +5665,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Tonight, I will steal away your heart.</t>
+          <t>Tonight, I will steal away your heart. (80% accuracy up)</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
@@ -5795,11 +5679,7 @@
           <t>Tonight, I will steal away your heart (Accuracy +80%.).</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5853,7 +5733,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>A support item used by people who can't swim.</t>
+          <t>A support item used by people who can't swim. (cures freeze)</t>
         </is>
       </c>
       <c r="E151" t="inlineStr"/>
@@ -5867,11 +5747,7 @@
           <t>A support item used by people who can't swim (Cure Freeze).</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6061,7 +5937,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Rice-based liquor aged for more than three years.</t>
+          <t>Rice-based liquor aged for more than three years. (TP +50, 50% Berserk)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -6075,11 +5951,7 @@
           <t>Rice-based liquor aged for more than three years (+50% ATK).</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6099,7 +5971,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>For nailing uncooperative ogres to the ground.</t>
+          <t>For nailing uncooperative ogres to the ground. (30% slow)</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -6113,11 +5985,7 @@
           <t>For nailing uncooperative ogres to the ground (Speed DOWN -60%.).</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6323,7 +6191,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Oil you can rub on a wound in place of salve. If you want.</t>
+          <t>Oil you can rub on a wound in place of salve. If you want. (HP +60, 20% evasion up)</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
@@ -6337,11 +6205,7 @@
           <t>Oil you can rub on a wound in place of salve. If you want (+20% EVA).</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6399,7 +6263,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Somebody shut it up!</t>
+          <t>Somebody shut it up! (cures sleep)</t>
         </is>
       </c>
       <c r="E166" t="inlineStr"/>
@@ -6413,11 +6277,7 @@
           <t>Somebody shut it up! (Cure Sleep).</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -6437,7 +6297,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Looks like that's a YES. (HP +200, sleep 75%)</t>
+          <t>Looks like that's a YES. (HP +200, 75% sleep)</t>
         </is>
       </c>
       <c r="E167" t="inlineStr"/>
@@ -6509,7 +6369,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Huge poisonous spike plucked from a tarasque's back.</t>
+          <t>Huge poisonous spike plucked from a tarasque's back. (35% poison)</t>
         </is>
       </c>
       <c r="E169" t="inlineStr"/>
@@ -6523,11 +6383,7 @@
           <t>Huge poisonous spike plucked from a tarasque's back (75% Poison).</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -6657,7 +6513,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Fake version of Alexandrite Cat's Eye.</t>
+          <t>Fake version of Alexandrite Cat's Eye. (30% accuracy up)</t>
         </is>
       </c>
       <c r="E173" t="inlineStr"/>
@@ -6671,11 +6527,7 @@
           <t>Fake version of Alexandrite Cat's Eye (Accuracy +30%.).</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -6832,7 +6684,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>You were forced to buy it at 5x the market price. I could cry. (sleep 90%)</t>
+          <t>You were forced to buy it at 5x the market price. I could cry. (90% sleep)</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
@@ -6866,7 +6718,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Unfortunately, it's a one-way ticket.</t>
+          <t>Unfortunately, it's a one-way ticket. (10% petrifying)</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
@@ -6880,11 +6732,7 @@
           <t>Unfortunately, it's a one-way ticket (Inflict Curse (40% chance).).</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6904,7 +6752,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Apparently it'll send you to another world with just one sip (it's poison).</t>
+          <t>It'll send you to another world with just one sip (it's poison). (30% instakill)</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
@@ -6921,7 +6769,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -6943,7 +6791,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Still a step or two away from being a salad.</t>
+          <t>Still a step or two away from being a salad. (20% Divine Shield)</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
@@ -6957,11 +6805,7 @@
           <t>Still a step or two away from being a salad.</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -7015,7 +6859,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Said to bring its holder happiness.</t>
+          <t>Said to bring its holder happiness. (30% Insurance, 30% evasion up)</t>
         </is>
       </c>
       <c r="E183" t="inlineStr"/>
@@ -7029,11 +6873,7 @@
           <t>Said to bring its holder happiness (+30% EVA).</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -7053,7 +6893,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Honestly, just cut me some slack.</t>
+          <t>Honestly, just cut me some slack. (15% petrifying)</t>
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
@@ -7067,11 +6907,7 @@
           <t>Honestly, just cut me some slack (Inflict Curse (30% chance).).</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -7091,7 +6927,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>It says it's lucky. You can't believe everything you read, now can you?</t>
+          <t>It says it's lucky. You can't believe everything you read, now can you? (15% silence)</t>
         </is>
       </c>
       <c r="E185" t="inlineStr"/>
@@ -7106,11 +6942,7 @@
 (30% Silence)</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -7130,7 +6962,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>A letter that simply says: You are my fire. My one desire.</t>
+          <t>A letter that simply says: You are my fire. My one desire. (50% accuracy up)</t>
         </is>
       </c>
       <c r="E186" t="inlineStr"/>
@@ -7144,11 +6976,7 @@
           <t>A letter that simply says: You are my fire. My one desire (Accuracy +50%.).</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -7168,7 +6996,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>The prompt asks, who's your personal hero? I wrote, 'Me.'</t>
+          <t>The prompt asks, who's your personal hero? I wrote, 'Me.' (80% Berserk)</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
@@ -7182,11 +7010,7 @@
           <t>The prompt asks, who's your personal hero? I wrote, 'Me.' (+80% ATK).</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -7206,7 +7030,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Tiger scroll filled with innermost secrets of martial arts.</t>
+          <t>Tiger scroll filled with innermost secrets of martial arts. (30% ATK up)</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
@@ -7220,11 +7044,7 @@
           <t>Tiger scroll filled with innermost secrets of martial arts (+30% ATK).</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -7244,7 +7064,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>The symbol of justice. Who needs bats, anyways?</t>
+          <t>The symbol of justice. Who needs bats, anyways? (50% ATK up)</t>
         </is>
       </c>
       <c r="E189" t="inlineStr"/>
@@ -7258,11 +7078,7 @@
           <t>The symbol of justice. Who needs bats, anyways? (+50% ATK).</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -7388,7 +7204,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Holy river water that contains all sorts of extracts. Extracts...</t>
+          <t>Holy river water that contains all sorts of extracts. Extracts... (TP +100, 75% stun)</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
@@ -7403,11 +7219,7 @@
 (+100 TP, 75% Blind)</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -7567,7 +7379,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>More of a snow acquaintance. A snowperson at any rate.</t>
+          <t>More of a snow acquaintance. A snowperson at any rate. (20% freeze)</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
@@ -7581,11 +7393,7 @@
           <t>More of a snow acquaintance. A snowperson at any rate (40% Freeze).</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -7923,7 +7731,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>An origami crane made with an exceedingly high number of folds.</t>
+          <t>An origami crane made with an exceedingly high number of folds. (60% party cure-all)</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
@@ -7937,11 +7745,7 @@
           <t>An origami crane made with an exceedingly high number of folds.</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -8101,7 +7905,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Dangerous box that shoots out needles when opened improperly.</t>
+          <t>Dangerous box that shoots out needles when opened improperly. (110 fixed damage)</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -8115,11 +7919,7 @@
           <t>Dangerous box that shoots out needles when opened improperly.</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -8207,7 +8007,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>A box full of contracts signed under threat of violence.</t>
+          <t>A box full of contracts signed under threat of violence. (party 150 fixed damage)</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
@@ -8221,11 +8021,7 @@
           <t>A box full of contracts signed under threat of violence.</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -8313,7 +8109,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>A sword with a bamboo grip. For some reason, the grip... reeks.</t>
+          <t>A sword with a bamboo grip. For some reason, the grip... reeks. (35% stun)</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
@@ -8327,11 +8123,7 @@
           <t>A sword with a bamboo grip. For some reason, the grip... reeks (50% Blind).</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -8385,7 +8177,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>A giant bloodshot eyeball. At least it's not moving.</t>
+          <t>A giant bloodshot eyeball. At least it's not moving. (35% paralysis)</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
@@ -8399,11 +8191,7 @@
           <t>A giant bloodshot eyeball. At least it's not moving (50% Paralysis).</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -8423,7 +8211,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>A chain that's been worn down by too much grinding. Kinda like my ex.</t>
+          <t>A chain worn down by too much grinding. Kinda like my ex. (15 fixed damage)</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
@@ -8439,7 +8227,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -8563,7 +8351,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Despite its not having a head, you swear you've heard it giggle.</t>
+          <t>Despite its not having a head, you swear you've heard it giggle. (22% paralysis)</t>
         </is>
       </c>
       <c r="E226" t="inlineStr"/>
@@ -8577,11 +8365,7 @@
           <t>Despite its not having a head, you swear you've heard it giggle (35% Paralysis).</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -8601,7 +8385,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Doll that changes to look just like you when you press its nose.</t>
+          <t>Doll that changes to look just like you when you press its nose. (30% 1 clone)</t>
         </is>
       </c>
       <c r="E227" t="inlineStr"/>
@@ -8615,11 +8399,7 @@
           <t>Doll that changes to look just like you when you press its nose.</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -8775,7 +8555,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Every time you look at it, the people are in different poses.</t>
+          <t>Every time you look at it, the people are in different poses. (15% silence)</t>
         </is>
       </c>
       <c r="E232" t="inlineStr"/>
@@ -8789,11 +8569,7 @@
           <t>Every time you look at it, the people are in different poses (30% Silence).</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -8813,7 +8589,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>A primal scream that resounds through the natural world.</t>
+          <t>A primal scream that resounds through the natural world. (20% stun)</t>
         </is>
       </c>
       <c r="E233" t="inlineStr"/>
@@ -8827,11 +8603,7 @@
           <t>A primal scream that resounds through the natural world (40% Blind).</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -8987,7 +8759,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Low-tech but reliable way to warm up.</t>
+          <t>Low-tech but reliable way to warm up. (cures freeze)</t>
         </is>
       </c>
       <c r="E238" t="inlineStr"/>
@@ -9001,11 +8773,7 @@
           <t>Low-tech but reliable way to warm up (Cure Freeze).</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -9025,7 +8793,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Not for use indoors. DEFINITELY not for use in a vehicle!</t>
+          <t>Not for use indoors. DEFINITELY not for use in a vehicle! (15% instakill)</t>
         </is>
       </c>
       <c r="E239" t="inlineStr"/>
@@ -9039,11 +8807,7 @@
           <t>Not for use indoors. DEFINITELY not for use in a vehicle! (30% Death).</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -9097,7 +8861,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Used for voodoo curses. Picture your enemy, and give it your all!</t>
+          <t>Used for voodoo curses. Picture your enemy, and give it your all! (12% stun)</t>
         </is>
       </c>
       <c r="E241" t="inlineStr"/>
@@ -9111,11 +8875,7 @@
           <t>Used for voodoo curses. Picture your enemy, and give it your all! (15% Blind).</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -9135,7 +8895,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Jelly infused with natural demon... stuff.</t>
+          <t>Jelly infused with natural demon... stuff. (10% poison, 10% silence)</t>
         </is>
       </c>
       <c r="E242" t="inlineStr"/>
@@ -9149,11 +8909,7 @@
           <t>Jelly infused with natural demon... stuff (20% Poison, 20% Silence).</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -9321,7 +9077,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Mist that covers your skin in glossy beads.</t>
+          <t>Mist that covers your skin in glossy beads. (TP +150, 30% freeze)</t>
         </is>
       </c>
       <c r="E247" t="inlineStr"/>
@@ -9335,11 +9091,7 @@
           <t>Mist that covers your skin in glossy beads (+150 TP, 30% Freeze).</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -9431,7 +9183,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>I'd like to think this is the cause for my weight gain...</t>
+          <t>I'd like to think this is the cause for my weight gain... (40% slow)</t>
         </is>
       </c>
       <c r="E250" t="inlineStr"/>
@@ -9445,11 +9197,7 @@
           <t>I'd like to think this is the cause for my weight gain.. (Speed DOWN -60%.).</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -9542,7 +9290,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Collecting seven of these summons a dragon that grants your wishes.</t>
+          <t>Collect seven of these to summon a wish-granting dragon. (75% strips buffs)</t>
         </is>
       </c>
       <c r="E253" t="inlineStr"/>
@@ -9558,7 +9306,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -9618,7 +9366,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>It had to be removed due to cavity.</t>
+          <t>It had to be removed due to cavity. (35% poison)</t>
         </is>
       </c>
       <c r="E255" t="inlineStr"/>
@@ -9632,11 +9380,7 @@
           <t>It had to be removed due to cavity (60% Poison).</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -9656,7 +9400,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>A paralyzing claw that was cut to the quick.</t>
+          <t>A paralyzing claw that was cut to the quick. (35% paralysis)</t>
         </is>
       </c>
       <c r="E256" t="inlineStr"/>
@@ -9670,11 +9414,7 @@
           <t>A paralyzing claw that was cut to the quick (60% Paralysis).</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -9732,7 +9472,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>No-good apple that tempts women into strife.</t>
+          <t>No-good apple that tempts women into strife. (party TP +100, party 500 fixed damage)</t>
         </is>
       </c>
       <c r="E258" t="inlineStr"/>
@@ -9746,11 +9486,7 @@
           <t>No-good apple that tempts women into strife (Party: +100 TP).</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -9804,7 +9540,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Huge bell that wards off evil when run. Awkward to carry around.</t>
+          <t>Huge bell that wards off evil when run. Awkward to carry around. (20% party DEF up)</t>
         </is>
       </c>
       <c r="E260" t="inlineStr"/>
@@ -9818,11 +9554,7 @@
           <t>Huge bell that wards off evil when run. Awkward to carry around.</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -9842,7 +9574,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Water from a shrine that venerates a god of the land.</t>
+          <t>Water from a shrine that venerates a god of the land. (90% party cure-all)</t>
         </is>
       </c>
       <c r="E261" t="inlineStr"/>
@@ -9856,11 +9588,7 @@
           <t>Water from a shrine that venerates a god of the land.</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -9880,7 +9608,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Fruit goes in the dragon. This stuff comes out. Don't ask.</t>
+          <t>Fruit goes in the dragon. This stuff comes out. Don't ask. (TP +50, 40% Berserk)</t>
         </is>
       </c>
       <c r="E262" t="inlineStr"/>
@@ -9894,11 +9622,7 @@
           <t>Fruit goes in the dragon. This stuff comes out. Don't ask (+40% ATK).</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -9918,7 +9642,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Press it if you want peace at any cost. There may be consequences...</t>
+          <t>Press it for peace at any cost. There may be consequences... (90% strips buffs)</t>
         </is>
       </c>
       <c r="E263" t="inlineStr"/>
@@ -9934,7 +9658,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -9956,7 +9680,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Used by busy mommy dragons to keep their babies quiet. (sleep 20%)</t>
+          <t>Used by busy mommy dragons to keep their babies quiet. (20% sleep)</t>
         </is>
       </c>
       <c r="E264" t="inlineStr"/>
@@ -9990,7 +9714,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Tough enough to survive in a mouth full of dragon baby teeth. (sleep 40%)</t>
+          <t>Tough enough to survive in a mouth full of dragon baby teeth. (40% sleep)</t>
         </is>
       </c>
       <c r="E265" t="inlineStr"/>
@@ -10058,7 +9782,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>A strange substance that feels like nothingness when you touch it.</t>
+          <t>A strange substance that feels like nothingness when you touch it. (30% evasion up)</t>
         </is>
       </c>
       <c r="E267" t="inlineStr"/>
@@ -10072,11 +9796,7 @@
           <t>A strange substance that feels like nothingness when you touch it (+30% EVA).</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -10096,7 +9816,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Not for napping in. For hiding people taking naps. (HP +200, sleep 90%)</t>
+          <t>Not for napping in. For hiding people taking naps. (HP +200, 90% sleep)</t>
         </is>
       </c>
       <c r="E268" t="inlineStr"/>
@@ -10130,7 +9850,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>A mask that is just gold in color. Not all that glitters is gold.</t>
+          <t>A mask that is just gold in color. Not all that glitters is gold. (12% paralysis)</t>
         </is>
       </c>
       <c r="E269" t="inlineStr"/>
@@ -10144,11 +9864,7 @@
           <t>A mask that is just gold in color. Not all that glitters is gold (15% Paralysis).</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -10240,7 +9956,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Goodnight forever.</t>
+          <t>Goodnight forever. (20% instakill)</t>
         </is>
       </c>
       <c r="E272" t="inlineStr"/>
@@ -10254,11 +9970,7 @@
           <t>Goodnight forever (60% Death).</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -10384,7 +10096,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Dangerous! Do not touch! Deadly poison! Requires careful handling!</t>
+          <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! (15% instakill)</t>
         </is>
       </c>
       <c r="E276" t="inlineStr"/>
@@ -10398,11 +10110,7 @@
           <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! (40% Death).</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -10422,7 +10130,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! #2</t>
+          <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! #2 (20% instakill)</t>
         </is>
       </c>
       <c r="E277" t="inlineStr"/>
@@ -10436,11 +10144,7 @@
           <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! #2 (80% Death).</t>
         </is>
       </c>
-      <c r="H277" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -10460,7 +10164,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>A nice little rowboat. Cruise the river separating life and death.</t>
+          <t>A nice little rowboat. Cruise the river separating life and death. (30% instakill)</t>
         </is>
       </c>
       <c r="E278" t="inlineStr"/>
@@ -10474,11 +10178,7 @@
           <t>A nice little rowboat. Cruise the river separating life and death (95% Death).</t>
         </is>
       </c>
-      <c r="H278" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -10498,7 +10198,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Sweet mint immortali-tea. More relaxing than relaxation itself. (TP +35, sleep 25%)</t>
+          <t>Sweet mint immortali-tea. More relaxing than relaxation itself. (TP +35, 25% sleep)</t>
         </is>
       </c>
       <c r="E279" t="inlineStr"/>
@@ -10532,7 +10232,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>So much jealousy, it's visible to the naked eye.</t>
+          <t>So much jealousy, it's visible to the naked eye. (30% paralysis, 30% sleep)</t>
         </is>
       </c>
       <c r="E280" t="inlineStr"/>
@@ -10546,11 +10246,7 @@
           <t>So much jealousy, it's visible to the naked eye (30% Paralysis, 30% Sleep).</t>
         </is>
       </c>
-      <c r="H280" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -10604,7 +10300,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Bun that gives off the taste of the afterlife.</t>
+          <t>Bun that gives off the taste of the afterlife. (HP +60, 25% stun)</t>
         </is>
       </c>
       <c r="E282" t="inlineStr"/>
@@ -10618,11 +10314,7 @@
           <t>Bun that gives off the taste of the afterlife (+60 HP, 25% Blind).</t>
         </is>
       </c>
-      <c r="H282" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -10676,7 +10368,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>I really hope my photo's not on there.</t>
+          <t>I really hope my photo's not on there. (15% petrifying)</t>
         </is>
       </c>
       <c r="E284" t="inlineStr"/>
@@ -10690,11 +10382,7 @@
           <t>I really hope my photo's not on there (Inflict Curse (20% chance).).</t>
         </is>
       </c>
-      <c r="H284" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -10748,7 +10436,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>You'll want to stay away from the water this came from.</t>
+          <t>You'll want to stay away from the water this came from. (25% paralysis)</t>
         </is>
       </c>
       <c r="E286" t="inlineStr"/>
@@ -10762,11 +10450,7 @@
           <t>You'll want to stay away from the water this came from (50% Paralysis).</t>
         </is>
       </c>
-      <c r="H286" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -10854,7 +10538,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Living shadow that leaves and acts on its own.</t>
+          <t>Living shadow that leaves and acts on its own. (25% 2 clones)</t>
         </is>
       </c>
       <c r="E289" t="inlineStr"/>
@@ -10868,11 +10552,7 @@
           <t>Living shadow that leaves and acts on its own.</t>
         </is>
       </c>
-      <c r="H289" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -10892,7 +10572,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Toss it in to any potluck stew to instantly increase the chaos.</t>
+          <t>Toss it in to any potluck stew to instantly increase the chaos. (50 fixed damage)</t>
         </is>
       </c>
       <c r="E290" t="inlineStr"/>
@@ -10906,11 +10586,7 @@
           <t>Toss it in to any potluck stew to instantly increase the chaos.</t>
         </is>
       </c>
-      <c r="H290" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -10964,7 +10640,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Just ignore them.</t>
+          <t>Just ignore them. (20% silence)</t>
         </is>
       </c>
       <c r="E292" t="inlineStr"/>
@@ -10978,11 +10654,7 @@
           <t>Just ignore them (40% Silence).</t>
         </is>
       </c>
-      <c r="H292" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -11002,7 +10674,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Disembodied wrist. Scurries all over the floor like a cleaning robot.</t>
+          <t>Disembodied wrist. Scurries all over the floor like a cleaning robot. (30% stun)</t>
         </is>
       </c>
       <c r="E293" t="inlineStr"/>
@@ -11016,11 +10688,7 @@
           <t>Disembodied wrist. Scurries all over the floor like a cleaning robot (60% Blind).</t>
         </is>
       </c>
-      <c r="H293" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -11188,7 +10856,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Ice cream in a peach-shaped container.</t>
+          <t>Ice cream in a peach-shaped container. (TP +12, 20% freeze)</t>
         </is>
       </c>
       <c r="E298" t="inlineStr"/>
@@ -11202,11 +10870,7 @@
           <t>Ice cream in a peach-shaped container (+12 TP, 20% Freeze).</t>
         </is>
       </c>
-      <c r="H298" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -11226,7 +10890,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Sweet mixed drink popular with the ladies. (TP +24, sleep 20%)</t>
+          <t>Sweet mixed drink popular with the ladies. (TP +24, 20% sleep)</t>
         </is>
       </c>
       <c r="E299" t="inlineStr"/>
@@ -11328,7 +10992,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Sweet persimmons fumigated with sulfur for preservation. Tasty.</t>
+          <t>Sweet persimmons preserved with sulfur. Tasty. (TP +15, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E302" t="inlineStr"/>
@@ -11345,7 +11009,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>no room for (TP +15, cures 1 ailment): 89 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -11401,7 +11065,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Sushi wrapped in persimmon leaves. Don't eat the leaves, kiddo.</t>
+          <t>Sushi in persimmon leaves. Don't eat the leaves. (party HP +130, cancels Shadow Sew)</t>
         </is>
       </c>
       <c r="E304" t="inlineStr"/>
@@ -11418,7 +11082,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>no room for (party HP +130, cancels Shadow Sew): 99 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -11440,7 +11104,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Stew of bear-meat citatap with pukusakina and plenty of veggies.</t>
+          <t>Bear-meat citatap stew with pukusakina and veggies. (party HP +600, cures freeze)</t>
         </is>
       </c>
       <c r="E305" t="inlineStr"/>
@@ -11457,7 +11121,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -11479,7 +11143,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Bear soup that warms up your body.</t>
+          <t>Bear soup that warms up your body. (HP +200, cures freeze)</t>
         </is>
       </c>
       <c r="E306" t="inlineStr"/>
@@ -11493,11 +11157,7 @@
           <t>Bear soup that warms up your body (+200 HP, Cure Freeze).</t>
         </is>
       </c>
-      <c r="H306" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -11619,7 +11279,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Piping hot fried chicken. Ask before you add lemon juice, just to be safe.</t>
+          <t>Hot fried chicken. Ask before you add lemon juice. (HP +240, restores stats)</t>
         </is>
       </c>
       <c r="E310" t="inlineStr"/>
@@ -11636,7 +11296,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>no room for (HP +240, restores stats): 100 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -11828,7 +11488,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Fried lamb meatballs with strong coriander scent.</t>
+          <t>Fried lamb meatballs with strong coriander scent. (TP +50, 100% evasion up)</t>
         </is>
       </c>
       <c r="E316" t="inlineStr"/>
@@ -11842,11 +11502,7 @@
           <t>Fried lamb meatballs with strong coriander scent (+100% EVA).</t>
         </is>
       </c>
-      <c r="H316" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -11900,7 +11556,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Brave penguins gave their lives to bring you fuel and soap.</t>
+          <t>Brave penguins gave their lives to bring you fuel and soap. (80% evasion up)</t>
         </is>
       </c>
       <c r="E318" t="inlineStr"/>
@@ -11914,11 +11570,7 @@
           <t>Brave penguins gave their lives to bring you fuel and soap (+80% EVA).</t>
         </is>
       </c>
-      <c r="H318" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -11972,7 +11624,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Feel refreshed by the mint's cold and transcendent stimulation.</t>
+          <t>Feel refreshed by the mint's cold, transcendent stimulation. (HP +200, cures sleep)</t>
         </is>
       </c>
       <c r="E320" t="inlineStr"/>
@@ -11988,7 +11640,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -12384,7 +12036,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Supplement with a pungently strange odor.</t>
+          <t>Supplement with a pungently strange odor. (5% poison)</t>
         </is>
       </c>
       <c r="E332" t="inlineStr"/>
@@ -12398,11 +12050,7 @@
           <t>Supplement with a pungently strange odor (5% Poison).</t>
         </is>
       </c>
-      <c r="H332" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -12422,7 +12070,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Sketchy in over seven ways. Get it? Like seven colors of the rainbow!</t>
+          <t>Sketchy in over seven ways. Get it? Like seven colors of the rainbow! (10% stun)</t>
         </is>
       </c>
       <c r="E333" t="inlineStr"/>
@@ -12436,11 +12084,7 @@
           <t>Sketchy in over seven ways. Get it? Like seven colors of the rainbow! (10% Blind).</t>
         </is>
       </c>
-      <c r="H333" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -12460,7 +12104,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>All your exhaustion magically melts away.</t>
+          <t>All your exhaustion magically melts away. (20% Insurance)</t>
         </is>
       </c>
       <c r="E334" t="inlineStr"/>
@@ -12474,11 +12118,7 @@
           <t>All your exhaustion magically melts away.</t>
         </is>
       </c>
-      <c r="H334" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -12566,7 +12206,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Three delicious aspects of the dumpling, together on one skewer.</t>
+          <t>Three aspects of the dumpling on one skewer. (party HP +180, 60% party ATK up)</t>
         </is>
       </c>
       <c r="E337" t="inlineStr"/>
@@ -12582,7 +12222,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -12676,7 +12316,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Raw meat cut fine and called a steak. Consume with caution.</t>
+          <t>Raw meat cut fine and called a steak. Eat with caution. (HP/TP +2000, 95% 1 clone)</t>
         </is>
       </c>
       <c r="E340" t="inlineStr"/>
@@ -12692,7 +12332,7 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -12850,7 +12490,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>Glutinous steamed rice dish with big pieces of chestnut.</t>
+          <t>Glutinous steamed rice dish with big pieces of chestnut. (HP +515, 30% 1 clone)</t>
         </is>
       </c>
       <c r="E345" t="inlineStr"/>
@@ -12864,11 +12504,7 @@
           <t>Glutinous steamed rice dish with big pieces of chestnut (+515 HP).</t>
         </is>
       </c>
-      <c r="H345" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -12922,7 +12558,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>Seashell-shaped snack. Sally sells them by the seashore.</t>
+          <t>Seashell-shaped snack. Sally sells them by the seashore. (HP +135, 30% accuracy up)</t>
         </is>
       </c>
       <c r="E347" t="inlineStr"/>
@@ -12936,11 +12572,7 @@
           <t>Seashell-shaped snack. Sally sells them by the seashore (+135 HP).</t>
         </is>
       </c>
-      <c r="H347" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -12960,7 +12592,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>Solidified syrup and dry fruit. A hard candy for hard men.</t>
+          <t>Syrup and dry fruit. A hard candy for hard men. (party HP +165, restores stats)</t>
         </is>
       </c>
       <c r="E348" t="inlineStr"/>
@@ -12977,7 +12609,7 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>no room for (party HP +165, restores stats): 90 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -12999,7 +12631,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>A cake with a figurine in it. Whoever finds the little feller gets to be king.</t>
+          <t>Cake with a figurine. Whoever finds it gets to be king. (party HP +250, party TP +25)</t>
         </is>
       </c>
       <c r="E349" t="inlineStr"/>
@@ -13016,7 +12648,7 @@
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>no room for (party HP +250, party TP +25): 108 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -13072,7 +12704,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>Off the shelf or the classy kind? They're really not that different.</t>
+          <t>Off the shelf or classy? Really not that different. (HP +50, 50% accuracy up)</t>
         </is>
       </c>
       <c r="E351" t="inlineStr"/>
@@ -13088,7 +12720,7 @@
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -13110,7 +12742,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>Party pastry constructed of fruits, custard, and jelly.</t>
+          <t>Party pastry of fruits, custard, and jelly. (party TP +115, 70% party magic DEF up)</t>
         </is>
       </c>
       <c r="E352" t="inlineStr"/>
@@ -13126,7 +12758,7 @@
       </c>
       <c r="H352" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -13216,7 +12848,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>A cookie cut into a highly complex shape. Ooh, looks like Japan!</t>
+          <t>A cookie in a complex shape. Looks like Japan! (party HP +200, 60% party cure-all)</t>
         </is>
       </c>
       <c r="E355" t="inlineStr"/>
@@ -13232,7 +12864,7 @@
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -13288,7 +12920,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>Rice cracker covered in plenty of cayenne powder.</t>
+          <t>Rice cracker covered in plenty of cayenne powder. (HP +120, 25% Defender)</t>
         </is>
       </c>
       <c r="E357" t="inlineStr"/>
@@ -13302,11 +12934,7 @@
           <t>Rice cracker covered in plenty of cayenne powder (+120 HP).</t>
         </is>
       </c>
-      <c r="H357" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -13326,7 +12954,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>Just a cracker with tasty sauce, but dang, that's tasty.</t>
+          <t>Just a cracker with tasty sauce, but dang, that's tasty. (HP +240, 50% Defender)</t>
         </is>
       </c>
       <c r="E358" t="inlineStr"/>
@@ -13340,11 +12968,7 @@
           <t>Just a cracker with tasty sauce, but dang, that's tasty (+240 HP).</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -13364,7 +12988,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>Pre-chewed for convenience. Yum!</t>
+          <t>Pre-chewed for convenience. Yum! (HP +300, 70% Defender)</t>
         </is>
       </c>
       <c r="E359" t="inlineStr"/>
@@ -13378,11 +13002,7 @@
           <t>Pre-chewed for convenience. Yum! (+300 HP).</t>
         </is>
       </c>
-      <c r="H359" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -13436,7 +13056,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>Extremely smelly and rotten tofu.</t>
+          <t>Extremely smelly and rotten tofu. (HP +120, 90% silence)</t>
         </is>
       </c>
       <c r="E361" t="inlineStr"/>
@@ -13450,11 +13070,7 @@
           <t>Extremely smelly and rotten tofu (+120 HP, 90% Silence).</t>
         </is>
       </c>
-      <c r="H361" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -13686,7 +13302,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Eat a long candy, live a long life. It's just math.</t>
+          <t>Eat a long candy, live a long life. It's just math. (TP +150, 75% accuracy up)</t>
         </is>
       </c>
       <c r="E368" t="inlineStr"/>
@@ -13700,11 +13316,7 @@
           <t>Eat a long candy, live a long life. It's just math (+150 TP).</t>
         </is>
       </c>
-      <c r="H368" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -13724,7 +13336,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>An extremely rare, top-notch candy from the demon world.</t>
+          <t>Rare, top-notch candy from the demon world. (party HP/TP +666, 95% party cure-all)</t>
         </is>
       </c>
       <c r="E369" t="inlineStr"/>
@@ -13740,7 +13352,7 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -13762,7 +13374,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>Meatball patty with conspicuous chunks of onion.</t>
+          <t>Meatball patty with conspicuous chunks of onion. (HP +80, 35% ATK up)</t>
         </is>
       </c>
       <c r="E370" t="inlineStr"/>
@@ -13776,11 +13388,7 @@
           <t>Meatball patty with conspicuous chunks of onion (+35% ATK).</t>
         </is>
       </c>
-      <c r="H370" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -13800,7 +13408,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>Sunny-side up egg on a patty. When to break the yolk...?</t>
+          <t>Sunny-side up egg on a patty. When to break the yolk...? (HP +300, 75% ATK up)</t>
         </is>
       </c>
       <c r="E371" t="inlineStr"/>
@@ -13814,11 +13422,7 @@
           <t>Sunny-side up egg on a patty. When to break the yolk...? (+75% ATK).</t>
         </is>
       </c>
-      <c r="H371" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -13986,7 +13590,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>An ominous monaka in the shape of a coffin.</t>
+          <t>An ominous monaka in the shape of a coffin. (35% instakill)</t>
         </is>
       </c>
       <c r="E376" t="inlineStr"/>
@@ -14000,11 +13604,7 @@
           <t>An ominous monaka in the shape of a coffin (95% Death).</t>
         </is>
       </c>
-      <c r="H376" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -14024,7 +13624,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>Sesame, white bean paste, and... red bean paste!</t>
+          <t>Sesame, white bean paste, and... red bean paste! (HP +400, 75% accuracy up)</t>
         </is>
       </c>
       <c r="E377" t="inlineStr"/>
@@ -14038,11 +13638,7 @@
           <t>Sesame, white bean paste, and... red bean paste! (+400 HP).</t>
         </is>
       </c>
-      <c r="H377" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -14096,7 +13692,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>Bright macarons with an assortment of colors.</t>
+          <t>Bright macarons with an assortment of colors. (HP +150, 75% accuracy up)</t>
         </is>
       </c>
       <c r="E379" t="inlineStr"/>
@@ -14110,11 +13706,7 @@
           <t>Bright macarons with an assortment of colors (+150 HP).</t>
         </is>
       </c>
-      <c r="H379" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -14134,7 +13726,7 @@
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>Cookies for your iron abs.</t>
+          <t>Cookies for your iron abs. (HP +50, 75% DEF up)</t>
         </is>
       </c>
       <c r="E380" t="inlineStr"/>
@@ -14148,11 +13740,7 @@
           <t>Cookies for your iron abs (+75% DEF).</t>
         </is>
       </c>
-      <c r="H380" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -14172,7 +13760,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>Cake for your swole six-pack.</t>
+          <t>Cake for your swole six-pack. (HP +100, 50% ATK up)</t>
         </is>
       </c>
       <c r="E381" t="inlineStr"/>
@@ -14186,11 +13774,7 @@
           <t>Cake for your swole six-pack (+50% ATK).</t>
         </is>
       </c>
-      <c r="H381" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -14210,7 +13794,7 @@
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>Staple food on Planet Muscle. Go from ripped to jacked.</t>
+          <t>Staple food on Planet Muscle. Go from ripped to jacked. (HP +300, 75% max HP up)</t>
         </is>
       </c>
       <c r="E382" t="inlineStr"/>
@@ -14224,11 +13808,7 @@
           <t>Staple food on Planet Muscle. Go from ripped to jacked (+300 HP).</t>
         </is>
       </c>
-      <c r="H382" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -14248,7 +13828,7 @@
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>Apple drink. Sweet, spiked, or sparkling. (TP +55, sleep 10%)</t>
+          <t>Apple drink. Sweet, spiked, or sparkling. (TP +55, 10% sleep)</t>
         </is>
       </c>
       <c r="E383" t="inlineStr"/>
@@ -14282,7 +13862,7 @@
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>Mellow, rich, and just the right amount of bitter. (TP +74, sleep 25%)</t>
+          <t>Mellow, rich, and just the right amount of bitter. (TP +74, 25% sleep)</t>
         </is>
       </c>
       <c r="E384" t="inlineStr"/>
@@ -14316,7 +13896,7 @@
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>Sultry spirit. The perfect apertif. (TP +140, sleep 35%)</t>
+          <t>Sultry spirit. The perfect apertif. (TP +140, 35% sleep)</t>
         </is>
       </c>
       <c r="E385" t="inlineStr"/>
@@ -14350,7 +13930,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>The oil of conversation. The philosophic wine. (TP +999, sleep 45%)</t>
+          <t>The oil of conversation. The philosophic wine. (TP +999, 45% sleep)</t>
         </is>
       </c>
       <c r="E386" t="inlineStr"/>
@@ -14384,7 +13964,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>You know you should stop but you just can't kelp yourself.</t>
+          <t>You know you should stop but you just can't kelp yourself. (TP +20, 40% silence)</t>
         </is>
       </c>
       <c r="E387" t="inlineStr"/>
@@ -14398,11 +13978,7 @@
           <t>You know you should stop but you just can't kelp yourself (+20 TP, 40% Silence).</t>
         </is>
       </c>
-      <c r="H387" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -14422,7 +13998,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>Sandfish simmered in sugar and soy sauce.</t>
+          <t>Sandfish simmered in sugar and soy sauce. (TP +30, 60% silence)</t>
         </is>
       </c>
       <c r="E388" t="inlineStr"/>
@@ -14436,11 +14012,7 @@
           <t>Sandfish simmered in sugar and soy sauce (+30 TP, 60% Silence).</t>
         </is>
       </c>
-      <c r="H388" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -14460,7 +14032,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>If you get served this without a warning, you're the butt of a joke.</t>
+          <t>Served without a warning, you're the butt of a joke. (TP +40, 60% silence)</t>
         </is>
       </c>
       <c r="E389" t="inlineStr"/>
@@ -14477,7 +14049,7 @@
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -14499,7 +14071,7 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>Bad looks and worse texture but weirdly addictive.</t>
+          <t>Bad looks and worse texture but weirdly addictive. (TP +50, 60% silence)</t>
         </is>
       </c>
       <c r="E390" t="inlineStr"/>
@@ -14513,11 +14085,7 @@
           <t>Bad looks and worse texture but weirdly addictive (+50 TP, 60% Silence).</t>
         </is>
       </c>
-      <c r="H390" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -14537,7 +14105,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>Flatten an octopus and this is what you get. There's plenty to go around.</t>
+          <t>A flattened octopus. Plenty to go around. (party HP +160, 20% party magic DEF up)</t>
         </is>
       </c>
       <c r="E391" t="inlineStr"/>
@@ -14554,7 +14122,7 @@
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -14576,7 +14144,7 @@
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>Rice with big ol' chunks of tentacle.</t>
+          <t>Rice with big ol' chunks of tentacle. (HP +400, 50% ATK up)</t>
         </is>
       </c>
       <c r="E392" t="inlineStr"/>
@@ -14590,11 +14158,7 @@
           <t>Rice with big ol' chunks of tentacle (+50% ATK).</t>
         </is>
       </c>
-      <c r="H392" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -14784,7 +14348,7 @@
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>Spiral sweet soaked in sugary syrup.</t>
+          <t>Spiral sweet soaked in sugary syrup. (TP +98, 50% accuracy up)</t>
         </is>
       </c>
       <c r="E398" t="inlineStr"/>
@@ -14798,11 +14362,7 @@
           <t>Spiral sweet soaked in sugary syrup (+98 TP).</t>
         </is>
       </c>
-      <c r="H398" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -15060,7 +14620,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>Red bean bun baked with fine gold wheat. Diabetics should avoid it.</t>
+          <t>Red bean bun of fine gold wheat. Diabetics should avoid it. (HP +400, 80% Defender)</t>
         </is>
       </c>
       <c r="E406" t="inlineStr"/>
@@ -15076,7 +14636,7 @@
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -15170,7 +14730,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Potato chips that'll blow your top.</t>
+          <t>Potato chips that'll blow your top. (40% ATK up, 70% stun)</t>
         </is>
       </c>
       <c r="E409" t="inlineStr"/>
@@ -15184,11 +14744,7 @@
           <t>Potato chips that'll blow your top (+40% ATK).</t>
         </is>
       </c>
-      <c r="H409" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -15310,7 +14866,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>A candy so sweet it will cause your brain to melt.</t>
+          <t>A candy so sweet it will cause your brain to melt. (HP +300, 30% silence)</t>
         </is>
       </c>
       <c r="E413" t="inlineStr"/>
@@ -15324,11 +14880,7 @@
           <t>A candy so sweet it will cause your brain to melt (+300 HP, 30% Silence).</t>
         </is>
       </c>
-      <c r="H413" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -15348,7 +14900,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>So spicy it makes your eyes hurt.</t>
+          <t>So spicy it makes your eyes hurt. (25% paralysis)</t>
         </is>
       </c>
       <c r="E414" t="inlineStr"/>
@@ -15362,11 +14914,7 @@
           <t>So spicy it makes your eyes hurt (25% Paralysis).</t>
         </is>
       </c>
-      <c r="H414" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -15386,7 +14934,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>Eat it and you'll sweat from every orifice you've got.</t>
+          <t>Eat it and you'll sweat from every orifice you've got. (HP +50, cures freeze)</t>
         </is>
       </c>
       <c r="E415" t="inlineStr"/>
@@ -15400,11 +14948,7 @@
           <t>Eat it and you'll sweat from every orifice you've got (+50 HP, Cure Freeze).</t>
         </is>
       </c>
-      <c r="H415" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -15424,7 +14968,7 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>First-timers will lose consciousness due to the spice.</t>
+          <t>First-timers will lose consciousness due to the spice. (HP/TP +75, 15% paralysis)</t>
         </is>
       </c>
       <c r="E416" t="inlineStr"/>
@@ -15438,11 +14982,7 @@
           <t>First-timers will lose consciousness due to the spice (+75 HP/TP, 15% Paralysis).</t>
         </is>
       </c>
-      <c r="H416" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -15462,7 +15002,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>So spicy, it's out of this world. Just one phone call and they'll deliver.</t>
+          <t>So spicy it's out of this world. One call and they deliver. (HP +400, 80% silence)</t>
         </is>
       </c>
       <c r="E417" t="inlineStr"/>
@@ -15479,7 +15019,7 @@
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -15777,7 +15317,7 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>The mushroom formerly known as matsutake. They're... fine.</t>
+          <t>The mushroom formerly known as matsutake. They're... fine. (25% Divine Shield)</t>
         </is>
       </c>
       <c r="E426" t="inlineStr"/>
@@ -15791,11 +15331,7 @@
           <t>The mushroom formerly known as matsutake. They're... fine.</t>
         </is>
       </c>
-      <c r="H426" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -15815,7 +15351,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Yellow with red spots. Eat it, and you might get bigger.</t>
+          <t>Yellow with red spots. Eat it, and you might get bigger. (50% max HP up)</t>
         </is>
       </c>
       <c r="E427" t="inlineStr"/>
@@ -15829,11 +15365,7 @@
           <t>Yellow with red spots. Eat it, and you might get bigger.</t>
         </is>
       </c>
-      <c r="H427" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -15921,7 +15453,7 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Refrigerated agar with added beans and fruits.</t>
+          <t>Refrigerated agar with added beans and fruits. (TP +160, cures freeze)</t>
         </is>
       </c>
       <c r="E430" t="inlineStr"/>
@@ -15935,11 +15467,7 @@
           <t>Refrigerated agar with added beans and fruits (+160 TP, Cure Freeze).</t>
         </is>
       </c>
-      <c r="H430" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -16095,7 +15623,7 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>This sticky pudding is speckled with raisins. It's just pudding. Honestly.</t>
+          <t>Sticky pudding with raisins. Just pudding. Honestly. (HP +100, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E435" t="inlineStr"/>
@@ -16112,7 +15640,7 @@
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t>no room for (HP +100, cures 1 ailment): 101 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -16168,7 +15696,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Ol' reliable. You can't go wrong with bean paste.</t>
+          <t>Ol' reliable. You can't go wrong with bean paste. (TP +125, 65% Insurance)</t>
         </is>
       </c>
       <c r="E437" t="inlineStr"/>
@@ -16182,11 +15710,7 @@
           <t>Ol' reliable. You can't go wrong with bean paste (+125 TP).</t>
         </is>
       </c>
-      <c r="H437" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -16206,7 +15730,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Soup made wholly out of leftovers. Liver and let die!</t>
+          <t>Soup made of leftovers. Liver and let die! (party TP +10, 20% party cure-all)</t>
         </is>
       </c>
       <c r="E438" t="inlineStr"/>
@@ -16222,7 +15746,7 @@
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -16244,7 +15768,7 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>The unagi's not necessarily good, but the sauce is.</t>
+          <t>The unagi's not always good, but the sauce is. (party TP +25, 40% party cure-all)</t>
         </is>
       </c>
       <c r="E439" t="inlineStr"/>
@@ -16260,7 +15784,7 @@
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -16282,7 +15806,7 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Dead eels on rice. It's terrible, you wouldn't want any.</t>
+          <t>Dead eels on rice. You wouldn't want any. (party TP +50, 60% party cure-all)</t>
         </is>
       </c>
       <c r="E440" t="inlineStr"/>
@@ -16298,7 +15822,7 @@
       </c>
       <c r="H440" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -16320,7 +15844,7 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Sushi roll containing sticky, smelly, fermented soybeans. Yum...?</t>
+          <t>Sushi roll of sticky, smelly, fermented soybeans. Yum...? (HP/TP +30, 50% silence)</t>
         </is>
       </c>
       <c r="E441" t="inlineStr"/>
@@ -16337,7 +15861,7 @@
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -16359,7 +15883,7 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>You must be mindful of your surroundings when eating this.</t>
+          <t>You must be mindful of your surroundings when eating this. (HP/TP +60, 60% silence)</t>
         </is>
       </c>
       <c r="E442" t="inlineStr"/>
@@ -16373,11 +15897,7 @@
           <t>You must be mindful of your surroundings when eating this (+60 HP/TP, 60% Silence).</t>
         </is>
       </c>
-      <c r="H442" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -16397,7 +15917,7 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Extremely smelly... but somehow delicious.</t>
+          <t>Extremely smelly... but somehow delicious. (HP/TP +100, 70% silence)</t>
         </is>
       </c>
       <c r="E443" t="inlineStr"/>
@@ -16411,11 +15931,7 @@
           <t>Extremely smelly... but somehow delicious (+100 HP/TP, 70% Silence).</t>
         </is>
       </c>
-      <c r="H443" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -16435,7 +15951,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>Silky-smooth little fish, rich in calcium.</t>
+          <t>Silky-smooth little fish, rich in calcium. (HP +40, 30% DEF up)</t>
         </is>
       </c>
       <c r="E444" t="inlineStr"/>
@@ -16449,11 +15965,7 @@
           <t>Silky-smooth little fish, rich in calcium (+30% DEF).</t>
         </is>
       </c>
-      <c r="H444" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -16473,7 +15985,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>Somewhat grotesque when the fish has the face of a man.</t>
+          <t>Somewhat grotesque when the fish has the face of a man. (HP +100, 40% stun)</t>
         </is>
       </c>
       <c r="E445" t="inlineStr"/>
@@ -16487,11 +15999,7 @@
           <t>Somewhat grotesque when the fish has the face of a man (+100 HP, 40% Blind).</t>
         </is>
       </c>
-      <c r="H445" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -16511,7 +16019,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>Well dried bonito flakes.</t>
+          <t>Well dried bonito flakes. (HP +120, 60% DEF up)</t>
         </is>
       </c>
       <c r="E446" t="inlineStr"/>
@@ -16525,11 +16033,7 @@
           <t>Well dried bonito flakes (+60% DEF).</t>
         </is>
       </c>
-      <c r="H446" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -16549,7 +16053,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Bonito so dry it's a blunt weapon. The world's hardest food.</t>
+          <t>Bonito so dry it's a blunt weapon. The world's hardest food. (HP +200, 80% DEF up)</t>
         </is>
       </c>
       <c r="E447" t="inlineStr"/>
@@ -16563,11 +16067,7 @@
           <t>Bonito so dry it's a blunt weapon. The world's hardest food (+80% DEF).</t>
         </is>
       </c>
-      <c r="H447" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -16655,7 +16155,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Bitter jelly allegedly good for the skin. Not so great for the tortoise.</t>
+          <t>Bitter jelly good for the skin. Not so great for the tortoise. (cures all ailments)</t>
         </is>
       </c>
       <c r="E450" t="inlineStr"/>
@@ -16672,7 +16172,7 @@
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t>no room for (cures all ailments): 93 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -16694,7 +16194,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Genuine, honest, real turtle soup! Would I lie to you?</t>
+          <t>Genuine, real turtle soup! Would I lie to you? (cures all ailments, 40% max HP up)</t>
         </is>
       </c>
       <c r="E451" t="inlineStr"/>
@@ -16710,7 +16210,7 @@
       </c>
       <c r="H451" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -16732,7 +16232,7 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>Made in an earthenware pot at high temperature. Delicious but steep.</t>
+          <t>Made in an earthenware pot. Delicious but steep. (cures all ailments, TP +125)</t>
         </is>
       </c>
       <c r="E452" t="inlineStr"/>
@@ -16749,7 +16249,7 @@
       </c>
       <c r="H452" t="inlineStr">
         <is>
-          <t>no room for (cures all ailments, TP +125): 98 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -16805,7 +16305,7 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>Bento with only meat and rice. Get those veggies out of here!</t>
+          <t>Bento with only meat and rice. Get those veggies out of here! (HP +150, 50% ATK up)</t>
         </is>
       </c>
       <c r="E454" t="inlineStr"/>
@@ -16819,11 +16319,7 @@
           <t>Bento with only meat and rice. Get those veggies out of here! (+50% ATK).</t>
         </is>
       </c>
-      <c r="H454" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H454" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -16843,7 +16339,7 @@
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>Sukiyaki bento with super luxurious wagyu included.</t>
+          <t>Sukiyaki bento with super luxurious wagyu included. (HP +200, 70% ATK up)</t>
         </is>
       </c>
       <c r="E455" t="inlineStr"/>
@@ -16857,11 +16353,7 @@
           <t>Sukiyaki bento with super luxurious wagyu included (+70% ATK).</t>
         </is>
       </c>
-      <c r="H455" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -16881,7 +16373,7 @@
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>Steak bento so delicious it'll make you dizzy.</t>
+          <t>Steak bento so delicious it'll make you dizzy. (HP +400, 90% ATK up)</t>
         </is>
       </c>
       <c r="E456" t="inlineStr"/>
@@ -16895,11 +16387,7 @@
           <t>Steak bento so delicious it'll make you dizzy (+90% ATK).</t>
         </is>
       </c>
-      <c r="H456" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -16919,7 +16407,7 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>A liquid formed from the drool of the elusive nuko.</t>
+          <t>A liquid formed from the drool of the elusive nuko. (20% poison)</t>
         </is>
       </c>
       <c r="E457" t="inlineStr"/>
@@ -16933,11 +16421,7 @@
           <t>A liquid formed from the drool of the elusive nuko (60% Poison).</t>
         </is>
       </c>
-      <c r="H457" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -17025,7 +16509,7 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>Don't drink too much if you like your brain cells.</t>
+          <t>Don't drink too much if you like your brain cells. (TP +75, 20% instakill)</t>
         </is>
       </c>
       <c r="E460" t="inlineStr"/>
@@ -17039,11 +16523,7 @@
           <t>Don't drink too much if you like your brain cells (+75 TP).</t>
         </is>
       </c>
-      <c r="H460" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H460" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -17097,7 +16577,7 @@
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>Cheap and delicious. Sometimes filled with strawberry or pudding.</t>
+          <t>Cheap and delicious. Sometimes filled with pudding. (HP +135, cancels Shadow Sew)</t>
         </is>
       </c>
       <c r="E462" t="inlineStr"/>
@@ -17114,7 +16594,7 @@
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t>no room for (HP +135, cancels Shadow Sew): 95 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -17272,7 +16752,7 @@
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>If you don't handle it with care, the cream will spurt all over you.</t>
+          <t>Handle it with care, or the cream will spurt all over you. (HP +200, 25% DEF up)</t>
         </is>
       </c>
       <c r="E467" t="inlineStr"/>
@@ -17288,7 +16768,7 @@
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -17344,7 +16824,7 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>Triple-stack of pancakes smothered in sticky maple syrup.</t>
+          <t>Triple-stack of pancakes in sticky maple syrup. (party HP +180, 25% party ATK up)</t>
         </is>
       </c>
       <c r="E469" t="inlineStr"/>
@@ -17360,7 +16840,7 @@
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -17382,7 +16862,7 @@
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>It means white mountain. And yet, yellow cake. Y u do dis?</t>
+          <t>It means white mountain. And yet, yellow cake. Y u do dis? (HP +300, 25% accuracy up)</t>
         </is>
       </c>
       <c r="E470" t="inlineStr"/>
@@ -17396,11 +16876,7 @@
           <t>It means white mountain. And yet, yellow cake. Y u do dis? (+300 HP).</t>
         </is>
       </c>
-      <c r="H470" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H470" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -17420,7 +16896,7 @@
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>Sweetness and justice are synonymous.</t>
+          <t>Sweetness and justice are synonymous. (HP +400, 25% evasion up)</t>
         </is>
       </c>
       <c r="E471" t="inlineStr"/>
@@ -17434,11 +16910,7 @@
           <t>Sweetness and justice are synonymous (+25% EVA).</t>
         </is>
       </c>
-      <c r="H471" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -17458,7 +16930,7 @@
       </c>
       <c r="D472" t="inlineStr">
         <is>
-          <t>A multi-layered, doughy pie cake.</t>
+          <t>A multi-layered, doughy pie cake. (party HP +300, 25% party magic DEF up)</t>
         </is>
       </c>
       <c r="E472" t="inlineStr"/>
@@ -17472,11 +16944,7 @@
           <t>A multi-layered, doughy pie cake (Party: +300 HP).</t>
         </is>
       </c>
-      <c r="H472" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -17496,7 +16964,7 @@
       </c>
       <c r="D473" t="inlineStr">
         <is>
-          <t>A luxury item perfect for souvenirs or gift exchanges.</t>
+          <t>A luxury item perfect for souvenirs or gifts. (party TP +200, 40% party DEF up)</t>
         </is>
       </c>
       <c r="E473" t="inlineStr"/>
@@ -17512,7 +16980,7 @@
       </c>
       <c r="H473" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -17568,7 +17036,7 @@
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>Liquor brewed from millet. Its mature flavor can become a habit. (HP +125, sleep 40%)</t>
+          <t>Liquor brewed from millet. Its mature flavor can become a habit. (HP +125, 40% sleep)</t>
         </is>
       </c>
       <c r="E475" t="inlineStr"/>
@@ -17602,7 +17070,7 @@
       </c>
       <c r="D476" t="inlineStr">
         <is>
-          <t>The mascot creature of this chocolate has yet to be identified by science.</t>
+          <t>Its mascot creature has yet to be identified by science. (HP +165, 20% stun)</t>
         </is>
       </c>
       <c r="E476" t="inlineStr"/>
@@ -17619,7 +17087,7 @@
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -17641,7 +17109,7 @@
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>Canned whale. Slowly vanishing from shelves.</t>
+          <t>Canned whale. Slowly vanishing from shelves. (HP +200, 25% Divine Shield)</t>
         </is>
       </c>
       <c r="E477" t="inlineStr"/>
@@ -17655,11 +17123,7 @@
           <t>Canned whale. Slowly vanishing from shelves (+200 HP).</t>
         </is>
       </c>
-      <c r="H477" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H477" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -17717,7 +17181,7 @@
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>Simple hotpot of whale and mizuna.</t>
+          <t>Simple hotpot of whale and mizuna. (party HP +400, 60% party DEF up)</t>
         </is>
       </c>
       <c r="E479" t="inlineStr"/>
@@ -17731,11 +17195,7 @@
           <t>Simple hotpot of whale and mizuna (Party: +400 HP).</t>
         </is>
       </c>
-      <c r="H479" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -17789,7 +17249,7 @@
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>Filled with meat and veggies! Very delicious.</t>
+          <t>Filled with meat and veggies! Very delicious. (HP +120, cures freeze)</t>
         </is>
       </c>
       <c r="E481" t="inlineStr"/>
@@ -17803,11 +17263,7 @@
           <t>Filled with meat and veggies! Very delicious (+120 HP, Cure Freeze).</t>
         </is>
       </c>
-      <c r="H481" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H481" t="inlineStr"/>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -17827,7 +17283,7 @@
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>Warms your body to the core on a cold day.</t>
+          <t>Warms your body to the core on a cold day. (HP +180, cures freeze)</t>
         </is>
       </c>
       <c r="E482" t="inlineStr"/>
@@ -17841,11 +17297,7 @@
           <t>Warms your body to the core on a cold day (+180 HP, Cure Freeze).</t>
         </is>
       </c>
-      <c r="H482" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H482" t="inlineStr"/>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -17865,7 +17317,7 @@
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>Jelly made with copious amounts of slime.</t>
+          <t>Jelly made with copious amounts of slime. (10 fixed damage, 10% slow)</t>
         </is>
       </c>
       <c r="E483" t="inlineStr"/>
@@ -17879,11 +17331,7 @@
           <t>Jelly made with copious amounts of slime (Speed DOWN -20%.).</t>
         </is>
       </c>
-      <c r="H483" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H483" t="inlineStr"/>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -17903,7 +17351,7 @@
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>Made from only the gloopiest cuts of the slime.</t>
+          <t>Made from only the gloopiest cuts of the slime. (30 fixed damage, 5% slow)</t>
         </is>
       </c>
       <c r="E484" t="inlineStr"/>
@@ -17917,11 +17365,7 @@
           <t>Made from only the gloopiest cuts of the slime (Speed DOWN -10%.).</t>
         </is>
       </c>
-      <c r="H484" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H484" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -17941,7 +17385,7 @@
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>So chewy it'll tire out your jaw.</t>
+          <t>So chewy it'll tire out your jaw. (50 fixed damage, 20% slow)</t>
         </is>
       </c>
       <c r="E485" t="inlineStr"/>
@@ -17955,11 +17399,7 @@
           <t>So chewy it'll tire out your jaw (Speed DOWN -40%.).</t>
         </is>
       </c>
-      <c r="H485" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H485" t="inlineStr"/>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -17979,7 +17419,7 @@
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>Bavarian cream filled with tons of slime. Appetizing, isn't it?</t>
+          <t>Bavarian cream full of slime. Appetizing? (party 50 fixed damage, 75% strips buffs)</t>
         </is>
       </c>
       <c r="E486" t="inlineStr"/>
@@ -17995,7 +17435,7 @@
       </c>
       <c r="H486" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -18017,7 +17457,7 @@
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>Spray that turns you into a super sadist for a few minutes.</t>
+          <t>Spray that turns you into a super sadist for a few minutes. (50% Berserk)</t>
         </is>
       </c>
       <c r="E487" t="inlineStr"/>
@@ -18031,11 +17471,7 @@
           <t>Spray that turns you into a super sadist for a few minutes (+50% ATK).</t>
         </is>
       </c>
-      <c r="H487" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H487" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -18055,7 +17491,7 @@
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>The feeling of being foreign. You're a stranger in a strange land.</t>
+          <t>Feeling foreign. You're a stranger in a strange land. (75% Berserk, 75% stun)</t>
         </is>
       </c>
       <c r="E488" t="inlineStr"/>
@@ -18071,7 +17507,7 @@
       </c>
       <c r="H488" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -18093,7 +17529,7 @@
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>Can stuffed with dragon meat. Rare and expensive but a little smelly.</t>
+          <t>Canned dragon meat. Rare, expensive, a little smelly. (TP +150, cures all ailments)</t>
         </is>
       </c>
       <c r="E489" t="inlineStr"/>
@@ -18110,7 +17546,7 @@
       </c>
       <c r="H489" t="inlineStr">
         <is>
-          <t>no room for (TP +150, cures all ailments): 99 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -18132,7 +17568,7 @@
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>No alcohol until you're 21! (HP +75, sleep 30%)</t>
+          <t>No alcohol until you're 21! (HP +75, 30% sleep)</t>
         </is>
       </c>
       <c r="E490" t="inlineStr"/>
@@ -18166,7 +17602,7 @@
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>Some have never tried this sake, but none have tried it only once.</t>
+          <t>Some never tried this sake, but none tried it only once. (HP +150, 15% sleep)</t>
         </is>
       </c>
       <c r="E491" t="inlineStr"/>
@@ -18183,7 +17619,7 @@
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>no room for (HP +150, sleep 15%): 87 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -18205,7 +17641,7 @@
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>Powerful sake that intoxicates even heavy drinkers. Super harsh flavor.</t>
+          <t>Sake that intoxicates even heavy drinkers. Super harsh. (HP +300, 20% stun)</t>
         </is>
       </c>
       <c r="E492" t="inlineStr"/>
@@ -18222,7 +17658,7 @@
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -18244,7 +17680,7 @@
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>Port wine carefully aged for over a hundred years. (HP +400, sleep 20%)</t>
+          <t>Port wine carefully aged for over a hundred years. (HP +400, 20% sleep)</t>
         </is>
       </c>
       <c r="E493" t="inlineStr"/>
@@ -18346,7 +17782,7 @@
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>Dish made by shoving waterfowls into a dragon corpse.</t>
+          <t>Dish made by shoving waterfowls into a dragon corpse. (HP/TP +200, 50% paralysis)</t>
         </is>
       </c>
       <c r="E496" t="inlineStr"/>
@@ -18360,11 +17796,7 @@
           <t>Dish made by shoving waterfowls into a dragon corpse (+200 HP/TP, 50% Paralysis).</t>
         </is>
       </c>
-      <c r="H496" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H496" t="inlineStr"/>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -18384,7 +17816,7 @@
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>A huge, hard egg. It's unbreakable.</t>
+          <t>A huge, hard egg. It's unbreakable. (HP/TP +260, 25% evasion up)</t>
         </is>
       </c>
       <c r="E497" t="inlineStr"/>
@@ -18398,11 +17830,7 @@
           <t>A huge, hard egg. It's unbreakable (+25% EVA).</t>
         </is>
       </c>
-      <c r="H497" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H497" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -18456,7 +17884,7 @@
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>Cloying, syrupy drink.</t>
+          <t>Cloying, syrupy drink. (party HP/TP +200, restores stats)</t>
         </is>
       </c>
       <c r="E499" t="inlineStr"/>
@@ -18470,11 +17898,7 @@
           <t>Cloying, syrupy drink (Party: +250 HP/TP, Clear Debuffs).</t>
         </is>
       </c>
-      <c r="H499" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H499" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -18494,7 +17918,7 @@
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>Meat so tender that it melts at the touch.</t>
+          <t>Meat so tender that it melts at the touch. (25% poison)</t>
         </is>
       </c>
       <c r="E500" t="inlineStr"/>
@@ -18508,11 +17932,7 @@
           <t>Meat so tender that it melts at the touch (50% Poison).</t>
         </is>
       </c>
-      <c r="H500" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H500" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
@@ -18532,7 +17952,7 @@
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>Meat is most delicious when it's almost rotten... or so they say.</t>
+          <t>Meat is most delicious when it's almost rotten... or so they say. (35% poison)</t>
         </is>
       </c>
       <c r="E501" t="inlineStr"/>
@@ -18546,11 +17966,7 @@
           <t>Meat is most delicious when it's almost rotten... or so they say (70% Poison).</t>
         </is>
       </c>
-      <c r="H501" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H501" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -18570,7 +17986,7 @@
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>Primitive meat that shines suspiciously. Basically steroids in meat form.</t>
+          <t>Meat that shines suspiciously. Steroids in meat form. (50% poison, 40% paralysis)</t>
         </is>
       </c>
       <c r="E502" t="inlineStr"/>
@@ -18587,7 +18003,7 @@
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -18779,7 +18195,7 @@
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>Konpeito as big as your fist.</t>
+          <t>Konpeito as big as your fist. (party TP +400, 50% 2 clones)</t>
         </is>
       </c>
       <c r="E508" t="inlineStr"/>
@@ -18793,11 +18209,7 @@
           <t>Konpeito as big as your fist (Party: +400 TP).</t>
         </is>
       </c>
-      <c r="H508" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H508" t="inlineStr"/>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
@@ -18817,7 +18229,7 @@
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>Beverage squeezed out of an apple creature's insides.</t>
+          <t>Beverage squeezed out of an apple creature's insides. (HP/TP +100, 40% poison)</t>
         </is>
       </c>
       <c r="E509" t="inlineStr"/>
@@ -18831,11 +18243,7 @@
           <t>Beverage squeezed out of an apple creature's insides (+100 HP/TP, 40% Poison).</t>
         </is>
       </c>
-      <c r="H509" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H509" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -18855,7 +18263,7 @@
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>A candy with a whole appler trapped inside.</t>
+          <t>A candy with a whole appler trapped inside. (HP/TP +200, 80% poison)</t>
         </is>
       </c>
       <c r="E510" t="inlineStr"/>
@@ -18869,11 +18277,7 @@
           <t>A candy with a whole appler trapped inside (+200 HP/TP, 80% Poison).</t>
         </is>
       </c>
-      <c r="H510" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H510" t="inlineStr"/>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
@@ -18893,7 +18297,7 @@
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>Beverage squeezed out of a melon creature's insides.</t>
+          <t>Beverage squeezed out of a melon creature's insides. (HP/TP +100, 90% paralysis)</t>
         </is>
       </c>
       <c r="E511" t="inlineStr"/>
@@ -18907,11 +18311,7 @@
           <t>Beverage squeezed out of a melon creature's insides (+100 HP/TP, 90% Paralysis).</t>
         </is>
       </c>
-      <c r="H511" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H511" t="inlineStr"/>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
@@ -18931,7 +18331,7 @@
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>Unrelated to that anime character who lets people eat her face.</t>
+          <t>Unrelated to the anime girl whose face gets eaten. (HP/TP +200, 80% paralysis)</t>
         </is>
       </c>
       <c r="E512" t="inlineStr"/>
@@ -18948,7 +18348,7 @@
       </c>
       <c r="H512" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -18970,7 +18370,7 @@
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>Beverage squeezed out of a banana creature's insides.</t>
+          <t>Beverage squeezed out of a banana creature's insides. (HP/TP +100, 40% silence)</t>
         </is>
       </c>
       <c r="E513" t="inlineStr"/>
@@ -18984,11 +18384,7 @@
           <t>Beverage squeezed out of a banana creature's insides (+100 HP/TP, 40% Silence).</t>
         </is>
       </c>
-      <c r="H513" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H513" t="inlineStr"/>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
@@ -19008,7 +18404,7 @@
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>It's a big banana. Looks pretty sexy.</t>
+          <t>It's a big banana. Looks pretty sexy. (HP/TP +200, 80% silence)</t>
         </is>
       </c>
       <c r="E514" t="inlineStr"/>
@@ -19022,11 +18418,7 @@
           <t>It's a big banana. Looks pretty sexy (+200 HP/TP, 80% Silence).</t>
         </is>
       </c>
-      <c r="H514" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H514" t="inlineStr"/>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -19046,7 +18438,7 @@
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>A Fairy Mandra that's badly wounded.</t>
+          <t>A Fairy Mandra that's badly wounded. (10% stun)</t>
         </is>
       </c>
       <c r="E515" t="inlineStr"/>
@@ -19060,11 +18452,7 @@
           <t>A Fairy Mandra that's badly wounded (10% Blind).</t>
         </is>
       </c>
-      <c r="H515" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H515" t="inlineStr"/>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
@@ -19152,7 +18540,7 @@
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>The trefoil of a mandra, used as a graduation charm.</t>
+          <t>A mandra trefoil, used as a graduation charm. (party TP +150, 60% party magic DEF up)</t>
         </is>
       </c>
       <c r="E518" t="inlineStr"/>
@@ -19168,7 +18556,7 @@
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -19190,7 +18578,7 @@
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>Made by grinding up mandras.</t>
+          <t>Made by grinding up mandras. (99% silence, 99% freeze)</t>
         </is>
       </c>
       <c r="E519" t="inlineStr"/>
@@ -19204,11 +18592,7 @@
           <t>Made by grinding up mandras (95% Silence, 95% Freeze).</t>
         </is>
       </c>
-      <c r="H519" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H519" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -19228,7 +18612,7 @@
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>An Otherworld Mandra that's badly wounded.</t>
+          <t>An Otherworld Mandra that's badly wounded. (15% poison)</t>
         </is>
       </c>
       <c r="E520" t="inlineStr"/>
@@ -19242,11 +18626,7 @@
           <t>An Otherworld Mandra that's badly wounded (15% Poison).</t>
         </is>
       </c>
-      <c r="H520" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H520" t="inlineStr"/>
     </row>
     <row r="521">
       <c r="A521" t="inlineStr">
@@ -19334,7 +18714,7 @@
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>Too much of it will cause severe hallucinations. Not the good kind.</t>
+          <t>Too much of it will cause severe hallucinations. Not the good kind. (80% Defender)</t>
         </is>
       </c>
       <c r="E523" t="inlineStr"/>
@@ -19348,11 +18728,7 @@
           <t>Too much of it will cause severe hallucinations. Not the good kind.</t>
         </is>
       </c>
-      <c r="H523" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H523" t="inlineStr"/>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
@@ -19372,7 +18748,7 @@
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>Freshly squeezed mandra juice. Nice and pulpy.</t>
+          <t>Fresh-squeezed mandra juice. Nice and pulpy. (party HP/TP +2000, 90% party cure-all)</t>
         </is>
       </c>
       <c r="E524" t="inlineStr"/>
@@ -19388,7 +18764,7 @@
       </c>
       <c r="H524" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -19410,7 +18786,7 @@
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>Said to bring good fortune. Does anyone actually believe that?</t>
+          <t>Said to bring good fortune. Does anyone actually believe that? (party HP/TP +1000)</t>
         </is>
       </c>
       <c r="E525" t="inlineStr"/>
@@ -19424,11 +18800,7 @@
           <t>Said to bring good fortune. Does anyone actually believe that? (Party: +1000 HP/TP).</t>
         </is>
       </c>
-      <c r="H525" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H525" t="inlineStr"/>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
@@ -19618,7 +18990,7 @@
       </c>
       <c r="D531" t="inlineStr">
         <is>
-          <t>Made in an attempt to achieve sake supremacy. To sake-cceed.</t>
+          <t>Made to achieve sake supremacy. To sake-cceed. (HP/TP +50, cures all ailments)</t>
         </is>
       </c>
       <c r="E531" t="inlineStr"/>
@@ -19635,7 +19007,7 @@
       </c>
       <c r="H531" t="inlineStr">
         <is>
-          <t>no room for (HP/TP +50, cures all ailments): 92 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -19657,7 +19029,7 @@
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>The denizens of the world above say these pair well with tea.</t>
+          <t>Denizens of the world above say these pair well with tea. (TP +1000, 90% Insurance)</t>
         </is>
       </c>
       <c r="E532" t="inlineStr"/>
@@ -19673,7 +19045,7 @@
       </c>
       <c r="H532" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -19729,7 +19101,7 @@
       </c>
       <c r="D534" t="inlineStr">
         <is>
-          <t>Rice cake that crumbles from the outside as you eat it.</t>
+          <t>Rice cake that crumbles from the outside as you eat it. (TP +130, 75% Divine Shield)</t>
         </is>
       </c>
       <c r="E534" t="inlineStr"/>
@@ -19743,11 +19115,7 @@
           <t>Rice cake that crumbles from the outside as you eat it (+130 TP).</t>
         </is>
       </c>
-      <c r="H534" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H534" t="inlineStr"/>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -19767,7 +19135,7 @@
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>Precious, sweet-smelling beverage made of liquified mana crystals.</t>
+          <t>Sweet-smelling beverage of liquified mana crystals. (TP +999, cures all ailments)</t>
         </is>
       </c>
       <c r="E535" t="inlineStr"/>
@@ -19784,7 +19152,7 @@
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>no room for (TP +999, cures all ailments): 96 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -19806,7 +19174,7 @@
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>Dangerous drink that lights a fire in your loins. Yowch! That's hot!</t>
+          <t>Drink that lights a fire in your loins. Yowch! Hot! (HP +5000, 99% max HP up)</t>
         </is>
       </c>
       <c r="E536" t="inlineStr"/>
@@ -19822,7 +19190,7 @@
       </c>
       <c r="H536" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -19878,7 +19246,7 @@
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>The most treasured treasure of the Dragon Palace... cures Freeze.</t>
+          <t>The most treasured treasure of the Dragon Palace... cures Freeze. (cures freeze)</t>
         </is>
       </c>
       <c r="E538" t="inlineStr"/>
@@ -19892,11 +19260,7 @@
           <t>The most treasured treasure of the Dragon Palace... cures Freeze (Cure Freeze).</t>
         </is>
       </c>
-      <c r="H538" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H538" t="inlineStr"/>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -19916,7 +19280,7 @@
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>Tender green bud held by the former ruler of the world.</t>
+          <t>Tender green bud held by the former ruler of the world. (95% strips buffs)</t>
         </is>
       </c>
       <c r="E539" t="inlineStr"/>
@@ -19930,11 +19294,7 @@
           <t>Tender green bud held by the former ruler of the world.</t>
         </is>
       </c>
-      <c r="H539" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H539" t="inlineStr"/>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -20158,7 +19518,7 @@
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>A precious book depicting powerful bonds between men.</t>
+          <t>A precious book depicting powerful bonds between men. (50% silence)</t>
         </is>
       </c>
       <c r="E546" t="inlineStr"/>
@@ -20172,11 +19532,7 @@
           <t>A precious book depicting powerful bonds between men (95% Silence).</t>
         </is>
       </c>
-      <c r="H546" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H546" t="inlineStr"/>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">

</xml_diff>

<commit_message>
feat: item lines fit the battle bar
item lines fit the battle bar; party box test; docs for the screen
limits

201 item sentences reworded by hand (sheet ShortItems) so that sentence
+ (data) fits 70 characters. Test for the party skill box limit (the
overflowing line minus 3). Roadmap and project doc record the limits
measured on screen and the screens seen.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_item_text.xlsx
+++ b/mod_project/data_tables/qol_item_text.xlsx
@@ -769,7 +769,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Yakisoba noodle bread. Sells out very quickly. (HP/TP +20, cures 1 ailment)</t>
+          <t>Yakisoba noodle bread. Sells out fast. (HP/TP +20, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -808,7 +808,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Premium steak sandwich, luxury sauce. Extra deluxe. (HP/TP +30, cures all ailments)</t>
+          <t>Steak sandwich, luxury sauce. Deluxe. (HP/TP +30, cures all ailments)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -847,7 +847,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Spicy curry that would make even a Maharaja groan. (HP/TP +150, cures all ailments)</t>
+          <t>Curry to make a Maharaja groan. (HP/TP +150, cures all ailments)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -886,7 +886,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Legendary food. Whoever eats it falls in love. (HP/TP +1000, cures all ailments)</t>
+          <t>Legendary. Eat it and fall in love. (HP/TP +1000, cures all ailments)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Revive a fallen ally. Considerably bitter aftertaste. (revives at 10% HP)</t>
+          <t>Revive a fallen ally. Very bitter aftertaste. (revives at 10% HP)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -1109,7 +1109,11 @@
           <t>Revive a fallen ally. Considerably bitter aftertaste (Revive 30% HP).</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1368,7 +1372,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Highly nutritious, it heals HP and TP but is extremely bitter. (HP +50, TP +20)</t>
+          <t>Nutritious, heals HP and TP, but extremely bitter. (HP +50, TP +20)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -1407,7 +1411,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Tea with condensed bitterness. I hear it's an acquired taste... (HP +30, TP +40)</t>
+          <t>Condensed bitterness. An acquired taste, I hear... (HP +30, TP +40)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -1421,7 +1425,11 @@
           <t>Tea with condensed bitterness. I hear it's an acquired taste.. (+30 HP, +40 TP).</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1441,7 +1449,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Beard's special bento. Balanced, big enough to share. (party HP +75, party TP +25)</t>
+          <t>Beard's special bento, made to share. (party HP +75, party TP +25)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1480,7 +1488,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Peggy's eggy milk pudding. It's said to be legendary. (TP +30, 20% sleep)</t>
+          <t>Peggy's eggy milk pudding. Said to be legendary. (TP +30, 20% sleep)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1494,7 +1502,11 @@
           <t>Peggy's eggy milk pudding. It's said to be legendary (+30 TP, 20% Sleep).</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1514,7 +1526,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Kumaya Mangetsudo's anpan. Low-calorie, but still delicious. (HP/TP +20, 15% sleep)</t>
+          <t>Kumaya Mangetsudo's low-calorie, tasty anpan. (HP/TP +20, 15% sleep)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1621,7 +1633,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Mary Florina's rich milk collagen gel. (cures all ailments, restores stats)</t>
+          <t>Mary Florina's milk collagen gel. (cures all ailments, restores stats)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1733,7 +1745,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>An exciting new way to cheat death. Courtesy of the Peggy Company. (revives at 1% HP)</t>
+          <t>A new way to cheat death, by the Peggy Company. (revives at 1% HP)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1747,7 +1759,11 @@
           <t>An exciting new way to cheat death. Courtesy of the Peggy Company (Revive 100% HP).</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1767,7 +1783,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>A cure for anything, and plenty of it. (cures all ailments, restores stats)</t>
+          <t>A cure for anything, and plenty. (cures all ailments, restores stats)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1951,7 +1967,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>An aged icon that's heard prayers year after year. (cures all ailments)</t>
+          <t>An aged icon that's heard years of prayers. (cures all ailments)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -1965,7 +1981,11 @@
           <t>An aged icon that's heard prayers year after year (Cure All Ailments).</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1985,7 +2005,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>A gun shell left by one who gave up their life for revolution. (restores stats)</t>
+          <t>A shell left by one who died for the revolution. (restores stats)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -1999,7 +2019,11 @@
           <t>A gun shell left by one who gave up their life for revolution (Clear Debuffs).</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2019,7 +2043,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>A splendidly well-made futuristic metal. It's a bit lumpy. Weird. (150 steps)</t>
+          <t>A well-made futuristic metal. A bit lumpy. Weird. (150 steps)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -2033,7 +2057,11 @@
           <t>A splendidly well-made futuristic metal. It's a bit lumpy. Weird (Light 30 steps).</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2053,7 +2081,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>It scrambles your brain, and then you die. No coming back from that. (10% instakill)</t>
+          <t>It scrambles your brain, then you die. No coming back. (10% instakill)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -2067,7 +2095,11 @@
           <t>It scrambles your brain, and then you die. No coming back from that (25% Death).</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2087,7 +2119,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Inscribed with impressive wish-granting runes. (80% Divine Shield, 80% Insurance)</t>
+          <t>Wish-granting runes. Impressive. (80% Divine Shield, 80% Insurance)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -2101,7 +2133,11 @@
           <t>Inscribed with impressive wish-granting runes.</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2155,7 +2191,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Rock-hard cracker. Snack and emergency ration! (HP/TP +75, cancels Shadow Sew)</t>
+          <t>Rock-hard snack and emergency food! (HP/TP +75, cancels Shadow Sew)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2304,7 +2340,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Wind that brought spring to the underworld. (80% party ATK up, 80% party DEF up)</t>
+          <t>Spring wind of the underworld. (80% party ATK up, 80% party DEF up)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2584,7 +2620,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>When I peeked in, something peeked back... There's someone in there! (6% instakill)</t>
+          <t>I peeked in, it peeked back... Someone's in there! (6% instakill)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2598,7 +2634,11 @@
           <t>When I peeked in, something peeked back... There's someone in there! (25% Death).</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2656,7 +2696,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Might be usable in traditional medicine... if anything. (cancels Shadow Sew)</t>
+          <t>Maybe usable in traditional medicine... maybe. (cancels Shadow Sew)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2670,7 +2710,11 @@
           <t>Might be usable in traditional medicine... if anything (Cure Shadow Sew &amp; Bind).</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2860,7 +2904,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Whatever's under the breading, it's good and fried. (HP/TP +175, 75% Berserk)</t>
+          <t>Whatever's in the breading, it's good fried. (HP/TP +175, 75% Berserk)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3174,7 +3218,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Might's not all that makes right. Money does the trick too. (cures all ailments)</t>
+          <t>Might's not all that makes right. Money does too. (cures all ailments)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -3188,7 +3232,11 @@
           <t>Might's not all that makes right. Money does the trick too (Cure All Ailments).</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3208,7 +3256,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>I must immediately depart on a long, long journey. Don't look for me. (25% silence)</t>
+          <t>I must leave on a long, long journey. Don't look for me. (25% silence)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -3222,7 +3270,11 @@
           <t>I must immediately depart on a long, long journey. Don't look for me (50% Silence).</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3280,7 +3332,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>A red feather you receive after donating to a fundraiser. (TP +150, 75% Berserk)</t>
+          <t>A red feather you get for donating to a cause. (TP +150, 75% Berserk)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -3294,7 +3346,11 @@
           <t>A red feather you receive after donating to a fundraiser (+75% ATK).</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3417,7 +3473,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Down came the rain, but this web did not get washed out. (leaves the dungeon)</t>
+          <t>The rain came down, but this web stayed put. (leaves the dungeon)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -3431,7 +3487,11 @@
           <t>Down came the rain, but this web did not get washed out (Escape Dungeon).</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3451,7 +3511,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>One prick with this needle would be disastrous. Handle with care. (20% poison)</t>
+          <t>One prick would be disastrous. Handle with care. (20% poison)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -3465,7 +3525,11 @@
           <t>One prick with this needle would be disastrous. Handle with care (40% Poison).</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3485,7 +3549,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>A mirror that reveals the truth... You might not want to look. (15% stun)</t>
+          <t>A mirror that shows the truth... You may not want to look. (15% stun)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -3499,7 +3563,11 @@
           <t>A mirror that reveals the truth... You might not want to look (30% Blind).</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3799,7 +3867,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Clay used for handicraft in the heavens. Heh. They soil themselves. (10% 2 clones)</t>
+          <t>Clay of the heavens. Heh. They soil themselves. (10% 2 clones)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3813,7 +3881,11 @@
           <t>Clay used for handicraft in the heavens. Heh. They soil themselves.</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3833,7 +3905,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Vial of mysterious holy water. Tiny waves ripple at the top. (cures 1 ailment)</t>
+          <t>Mysterious holy water. Tiny waves ripple on top. (cures 1 ailment)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -3872,7 +3944,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Fried up in an iron pan. A steal at 3 million lira! (HP +50, 20% ATK up)</t>
+          <t>Pan-fried. A steal at 3 million lira! (HP +50, 20% ATK up)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -3886,7 +3958,11 @@
           <t>Fried up in an iron pan. A steal at 3 million lira! (+20% ATK).</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3906,7 +3982,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>There's no wind blowing, yet you can hear its sound. It cries Mary. (15% silence)</t>
+          <t>No wind blows, yet you hear its sound. It cries Mary. (15% silence)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -3920,7 +3996,11 @@
           <t>There's no wind blowing, yet you can hear its sound. It cries Mary (30% Silence).</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4012,7 +4092,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Just one drop will refresh constantly overworked eyes. (80% accuracy up)</t>
+          <t>One drop refreshes constantly overworked eyes. (80% accuracy up)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4026,7 +4106,11 @@
           <t>Just one drop will refresh constantly overworked eyes (Accuracy +80%.).</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4080,7 +4164,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Blowing or splashing water won't put out this fire. We didn't start it. (75 steps)</t>
+          <t>Blowing or water won't put it out. We didn't start it. (75 steps)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4095,7 +4179,11 @@
 (Light 15 steps)</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4187,7 +4275,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>The fruit, sadly, not the special event. Sweet and packed with energy. (TP +24)</t>
+          <t>The fruit, sadly, not the event. Sweet, packed with energy. (TP +24)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -4201,7 +4289,11 @@
           <t>The fruit, sadly, not the special event. Sweet and packed with energy (+24 TP).</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4221,7 +4313,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>If this waits back at base, someone's about to die. (TP +40, 30% instakill)</t>
+          <t>If it waits at base, someone's about to die. (TP +40, 30% instakill)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -4259,7 +4351,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>A pastry for the prosperous. Crumbles on your tongue. (party HP +100, party TP +40)</t>
+          <t>A pastry for the prosperous. Crumbly. (party HP +100, party TP +40)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -4273,7 +4365,11 @@
           <t>A pastry for the prosperous. Crumbles on your tongue (Party: +100 HP, +40 TP).</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4811,7 +4907,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>A skull from a secret rite. Grants wishes. (60% party ATK up, 30% party magic DEF up)</t>
+          <t>Rite skull. Grants wishes. (60% party ATK up, 30% party magic DEF up)</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4883,7 +4979,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>It makes a nice crunching sound when you bite into it. (revives at 35% HP)</t>
+          <t>Makes a nice crunch when you bite into it. (revives at 35% HP)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -4897,7 +4993,11 @@
           <t>It makes a nice crunching sound when you bite into it (Revive 35% HP).</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4917,7 +5017,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>A branch only some may pray to. It's twig-sclusive. (cures all ailments)</t>
+          <t>A branch only some may pray to. Twig-sclusive. (cures all ailments)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -4990,7 +5090,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Sandals that are no longer of any use. Might as well toss 'em. (15% evasion up)</t>
+          <t>Useless sandals. Might as well toss 'em. (15% evasion up)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5004,7 +5104,11 @@
           <t>Sandals that are no longer of any use. Might as well toss 'em (+15% EVA).</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5168,7 +5272,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Do YOU ever ruin your good cleaver on bone? Finally, there's help! (50% ATK up)</t>
+          <t>Ruined your good cleaver on bone? Finally, there's help! (50% ATK up)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5182,7 +5286,11 @@
           <t>Do YOU ever ruin your good cleaver on bone? Finally, there's help! (+50% ATK).</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5347,7 +5455,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>It might take... one more hit. Hit it baby one more time. (30 fixed damage)</t>
+          <t>One more hit... Hit it baby one more time. (30 fixed damage)</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5385,7 +5493,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Do the goggles switch her personality, or just add confidence...? (50% max HP up)</t>
+          <t>Do they switch her personality, or add confidence...? (50% max HP up)</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5563,7 +5671,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Eat this and you may die on the spot... or not at all. (90% instakill, TP +999)</t>
+          <t>Eat it and die on the spot... or never. (90% instakill, TP +999)</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5577,7 +5685,11 @@
           <t>Eat this and you may die on the spot... or not at all (+999 TP).</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5937,7 +6049,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Rice-based liquor aged for more than three years. (TP +50, 50% Berserk)</t>
+          <t>Rice liquor aged for more than three years. (TP +50, 50% Berserk)</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -5951,7 +6063,11 @@
           <t>Rice-based liquor aged for more than three years (+50% ATK).</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6191,7 +6307,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Oil you can rub on a wound in place of salve. If you want. (HP +60, 20% evasion up)</t>
+          <t>Oil for wounds instead of salve. If you want. (HP +60, 20% evasion up)</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
@@ -6205,7 +6321,11 @@
           <t>Oil you can rub on a wound in place of salve. If you want (+20% EVA).</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6684,7 +6804,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>You were forced to buy it at 5x the market price. I could cry. (90% sleep)</t>
+          <t>You were forced to buy it at 5x the price. I could cry. (90% sleep)</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
@@ -6698,7 +6818,11 @@
           <t>You were forced to buy it at 5x the market price. I could cry (90% Sleep).</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6752,7 +6876,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>It'll send you to another world with just one sip (it's poison). (30% instakill)</t>
+          <t>One sip sends you to another world (it's poison). (30% instakill)</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
@@ -6927,7 +7051,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>It says it's lucky. You can't believe everything you read, now can you? (15% silence)</t>
+          <t>It says it's lucky. Can't believe all you read, can you? (15% silence)</t>
         </is>
       </c>
       <c r="E185" t="inlineStr"/>
@@ -6942,7 +7066,11 @@
 (30% Silence)</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6962,7 +7090,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>A letter that simply says: You are my fire. My one desire. (50% accuracy up)</t>
+          <t>It simply says: You are my fire. My one desire. (50% accuracy up)</t>
         </is>
       </c>
       <c r="E186" t="inlineStr"/>
@@ -6976,7 +7104,11 @@
           <t>A letter that simply says: You are my fire. My one desire (Accuracy +50%.).</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6996,7 +7128,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>The prompt asks, who's your personal hero? I wrote, 'Me.' (80% Berserk)</t>
+          <t>Prompt: who's your personal hero? I wrote, 'Me.' (80% Berserk)</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
@@ -7010,7 +7142,11 @@
           <t>The prompt asks, who's your personal hero? I wrote, 'Me.' (+80% ATK).</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -7030,7 +7166,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Tiger scroll filled with innermost secrets of martial arts. (30% ATK up)</t>
+          <t>Tiger scroll of the innermost secrets of martial arts. (30% ATK up)</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
@@ -7044,7 +7180,11 @@
           <t>Tiger scroll filled with innermost secrets of martial arts (+30% ATK).</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -7204,7 +7344,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Holy river water that contains all sorts of extracts. Extracts... (TP +100, 75% stun)</t>
+          <t>Holy river water full of extracts. Extracts... (TP +100, 75% stun)</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
@@ -7219,7 +7359,11 @@
 (+100 TP, 75% Blind)</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -7595,7 +7739,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Good for massages and hair care and so on. (cancels Shadow Sew, restores stats)</t>
+          <t>For massages, hair care, etc. (cancels Shadow Sew, restores stats)</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
@@ -7609,7 +7753,11 @@
           <t>Good for massages and hair care and so on (Cure Shadow Sew).</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -7731,7 +7879,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>An origami crane made with an exceedingly high number of folds. (60% party cure-all)</t>
+          <t>An origami crane with a great many folds. (60% party cure-all)</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
@@ -7745,7 +7893,11 @@
           <t>An origami crane made with an exceedingly high number of folds.</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -7905,7 +8057,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Dangerous box that shoots out needles when opened improperly. (110 fixed damage)</t>
+          <t>Shoots out needles when opened improperly. (110 fixed damage)</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -7919,7 +8071,11 @@
           <t>Dangerous box that shoots out needles when opened improperly.</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -8007,7 +8163,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>A box full of contracts signed under threat of violence. (party 150 fixed damage)</t>
+          <t>Contracts signed under threat of violence. (party 150 fixed damage)</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
@@ -8021,7 +8177,11 @@
           <t>A box full of contracts signed under threat of violence.</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -8109,7 +8269,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>A sword with a bamboo grip. For some reason, the grip... reeks. (35% stun)</t>
+          <t>A sword with a bamboo grip. Somehow the grip... reeks. (35% stun)</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
@@ -8123,7 +8283,11 @@
           <t>A sword with a bamboo grip. For some reason, the grip... reeks (50% Blind).</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -8211,7 +8375,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>A chain worn down by too much grinding. Kinda like my ex. (15 fixed damage)</t>
+          <t>Worn down by too much grinding. Kinda like my ex. (15 fixed damage)</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
@@ -8351,7 +8515,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Despite its not having a head, you swear you've heard it giggle. (22% paralysis)</t>
+          <t>It has no head, yet you swear you've heard it giggle. (22% paralysis)</t>
         </is>
       </c>
       <c r="E226" t="inlineStr"/>
@@ -8365,7 +8529,11 @@
           <t>Despite its not having a head, you swear you've heard it giggle (35% Paralysis).</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -8385,7 +8553,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Doll that changes to look just like you when you press its nose. (30% 1 clone)</t>
+          <t>Press its nose and it changes to look just like you. (30% 1 clone)</t>
         </is>
       </c>
       <c r="E227" t="inlineStr"/>
@@ -8399,7 +8567,11 @@
           <t>Doll that changes to look just like you when you press its nose.</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -8555,7 +8727,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Every time you look at it, the people are in different poses. (15% silence)</t>
+          <t>Each time you look, the people are in different poses. (15% silence)</t>
         </is>
       </c>
       <c r="E232" t="inlineStr"/>
@@ -8569,7 +8741,11 @@
           <t>Every time you look at it, the people are in different poses (30% Silence).</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -8793,7 +8969,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Not for use indoors. DEFINITELY not for use in a vehicle! (15% instakill)</t>
+          <t>Not for indoors. DEFINITELY not for use in a vehicle! (15% instakill)</t>
         </is>
       </c>
       <c r="E239" t="inlineStr"/>
@@ -8807,7 +8983,11 @@
           <t>Not for use indoors. DEFINITELY not for use in a vehicle! (30% Death).</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -8861,7 +9041,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Used for voodoo curses. Picture your enemy, and give it your all! (12% stun)</t>
+          <t>For voodoo curses. Picture your enemy, give it your all! (12% stun)</t>
         </is>
       </c>
       <c r="E241" t="inlineStr"/>
@@ -8875,7 +9055,11 @@
           <t>Used for voodoo curses. Picture your enemy, and give it your all! (15% Blind).</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -9149,7 +9333,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>A boxful of crackin' chocolate. The ladies love it! (party TP +75, restores stats)</t>
+          <t>Crackin' chocolate. Ladies love it! (party TP +75, restores stats)</t>
         </is>
       </c>
       <c r="E249" t="inlineStr"/>
@@ -9163,7 +9347,11 @@
           <t>A boxful of crackin' chocolate. The ladies love it! (Party: +75 TP, Clear Debuffs).</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -9290,7 +9478,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Collect seven of these to summon a wish-granting dragon. (75% strips buffs)</t>
+          <t>Collect seven to summon a wish-granting dragon. (75% strips buffs)</t>
         </is>
       </c>
       <c r="E253" t="inlineStr"/>
@@ -9472,7 +9660,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>No-good apple that tempts women into strife. (party TP +100, party 500 fixed damage)</t>
+          <t>Tempts women into strife. (party TP +100, party 500 fixed damage)</t>
         </is>
       </c>
       <c r="E258" t="inlineStr"/>
@@ -9486,7 +9674,11 @@
           <t>No-good apple that tempts women into strife (Party: +100 TP).</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -9540,7 +9732,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Huge bell that wards off evil when run. Awkward to carry around. (20% party DEF up)</t>
+          <t>Huge bell that wards off evil. Awkward to carry. (20% party DEF up)</t>
         </is>
       </c>
       <c r="E260" t="inlineStr"/>
@@ -9554,7 +9746,11 @@
           <t>Huge bell that wards off evil when run. Awkward to carry around.</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -9574,7 +9770,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Water from a shrine that venerates a god of the land. (90% party cure-all)</t>
+          <t>Water from a shrine to a god of the land. (90% party cure-all)</t>
         </is>
       </c>
       <c r="E261" t="inlineStr"/>
@@ -9588,7 +9784,11 @@
           <t>Water from a shrine that venerates a god of the land.</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -9608,7 +9808,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Fruit goes in the dragon. This stuff comes out. Don't ask. (TP +50, 40% Berserk)</t>
+          <t>Fruit in the dragon, this out. Don't ask. (TP +50, 40% Berserk)</t>
         </is>
       </c>
       <c r="E262" t="inlineStr"/>
@@ -9622,7 +9822,11 @@
           <t>Fruit goes in the dragon. This stuff comes out. Don't ask (+40% ATK).</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -9642,7 +9846,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Press it for peace at any cost. There may be consequences... (90% strips buffs)</t>
+          <t>Peace at any cost. There may be consequences... (90% strips buffs)</t>
         </is>
       </c>
       <c r="E263" t="inlineStr"/>
@@ -9714,7 +9918,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Tough enough to survive in a mouth full of dragon baby teeth. (40% sleep)</t>
+          <t>Tough enough for a mouth full of dragon baby teeth. (40% sleep)</t>
         </is>
       </c>
       <c r="E265" t="inlineStr"/>
@@ -9728,7 +9932,11 @@
           <t>Tough enough to survive in a mouth full of dragon baby teeth (40% Sleep).</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -9782,7 +9990,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>A strange substance that feels like nothingness when you touch it. (30% evasion up)</t>
+          <t>Strange substance. Touching it feels like nothing. (30% evasion up)</t>
         </is>
       </c>
       <c r="E267" t="inlineStr"/>
@@ -9796,7 +10004,11 @@
           <t>A strange substance that feels like nothingness when you touch it (+30% EVA).</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -9816,7 +10028,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Not for napping in. For hiding people taking naps. (HP +200, 90% sleep)</t>
+          <t>Not for napping in. For hiding nappers. (HP +200, 90% sleep)</t>
         </is>
       </c>
       <c r="E268" t="inlineStr"/>
@@ -9830,7 +10042,11 @@
           <t>Not for napping in. For hiding people taking naps (+200 HP, 90% Sleep).</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -9850,7 +10066,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>A mask that is just gold in color. Not all that glitters is gold. (12% paralysis)</t>
+          <t>Just gold in color. Not all that glitters is gold. (12% paralysis)</t>
         </is>
       </c>
       <c r="E269" t="inlineStr"/>
@@ -9864,7 +10080,11 @@
           <t>A mask that is just gold in color. Not all that glitters is gold (15% Paralysis).</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -10096,7 +10316,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! (15% instakill)</t>
+          <t>Dangerous! Do not touch! Deadly poison! (15% instakill)</t>
         </is>
       </c>
       <c r="E276" t="inlineStr"/>
@@ -10110,7 +10330,11 @@
           <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! (40% Death).</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -10130,7 +10354,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! #2 (20% instakill)</t>
+          <t>Dangerous! Do not touch! Deadly poison! #2 (20% instakill)</t>
         </is>
       </c>
       <c r="E277" t="inlineStr"/>
@@ -10144,7 +10368,11 @@
           <t>Dangerous! Do not touch! Deadly poison! Requires careful handling! #2 (80% Death).</t>
         </is>
       </c>
-      <c r="H277" t="inlineStr"/>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -10164,7 +10392,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>A nice little rowboat. Cruise the river separating life and death. (30% instakill)</t>
+          <t>Nice rowboat. Cruise the river between life and death. (30% instakill)</t>
         </is>
       </c>
       <c r="E278" t="inlineStr"/>
@@ -10178,7 +10406,11 @@
           <t>A nice little rowboat. Cruise the river separating life and death (95% Death).</t>
         </is>
       </c>
-      <c r="H278" t="inlineStr"/>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -10198,7 +10430,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Sweet mint immortali-tea. More relaxing than relaxation itself. (TP +35, 25% sleep)</t>
+          <t>Sweet mint immortali-tea. Beyond relaxing. (TP +35, 25% sleep)</t>
         </is>
       </c>
       <c r="E279" t="inlineStr"/>
@@ -10212,7 +10444,11 @@
           <t>Sweet mint immortali-tea. More relaxing than relaxation itself (+35 TP, 25% Sleep).</t>
         </is>
       </c>
-      <c r="H279" t="inlineStr"/>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -10232,7 +10468,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>So much jealousy, it's visible to the naked eye. (30% paralysis, 30% sleep)</t>
+          <t>Jealousy so thick you can see it. (30% paralysis, 30% sleep)</t>
         </is>
       </c>
       <c r="E280" t="inlineStr"/>
@@ -10246,7 +10482,11 @@
           <t>So much jealousy, it's visible to the naked eye (30% Paralysis, 30% Sleep).</t>
         </is>
       </c>
-      <c r="H280" t="inlineStr"/>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -10436,7 +10676,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>You'll want to stay away from the water this came from. (25% paralysis)</t>
+          <t>Stay away from the water this came from. (25% paralysis)</t>
         </is>
       </c>
       <c r="E286" t="inlineStr"/>
@@ -10450,7 +10690,11 @@
           <t>You'll want to stay away from the water this came from (50% Paralysis).</t>
         </is>
       </c>
-      <c r="H286" t="inlineStr"/>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -10572,7 +10816,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Toss it in to any potluck stew to instantly increase the chaos. (50 fixed damage)</t>
+          <t>Toss it in any potluck stew for instant chaos. (50 fixed damage)</t>
         </is>
       </c>
       <c r="E290" t="inlineStr"/>
@@ -10586,7 +10830,11 @@
           <t>Toss it in to any potluck stew to instantly increase the chaos.</t>
         </is>
       </c>
-      <c r="H290" t="inlineStr"/>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -10674,7 +10922,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Disembodied wrist. Scurries all over the floor like a cleaning robot. (30% stun)</t>
+          <t>Disembodied wrist. Scurries about like a cleaning robot. (30% stun)</t>
         </is>
       </c>
       <c r="E293" t="inlineStr"/>
@@ -10688,7 +10936,11 @@
           <t>Disembodied wrist. Scurries all over the floor like a cleaning robot (60% Blind).</t>
         </is>
       </c>
-      <c r="H293" t="inlineStr"/>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -10924,7 +11176,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Peach-shaped bun eaten in times of celebration. (TP +36, cures 1 ailment)</t>
+          <t>Peach-shaped bun for celebrations. (TP +36, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E300" t="inlineStr"/>
@@ -10938,7 +11190,11 @@
           <t>Peach-shaped bun eaten in times of celebration (+36 TP, Cure 1 Ailment).</t>
         </is>
       </c>
-      <c r="H300" t="inlineStr"/>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -10992,7 +11248,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Sweet persimmons preserved with sulfur. Tasty. (TP +15, cures 1 ailment)</t>
+          <t>Sweet sulfur-preserved persimmons. Tasty. (TP +15, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E302" t="inlineStr"/>
@@ -11065,7 +11321,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Sushi in persimmon leaves. Don't eat the leaves. (party HP +130, cancels Shadow Sew)</t>
+          <t>Don't eat the persimmon leaves. (party HP +130, cancels Shadow Sew)</t>
         </is>
       </c>
       <c r="E304" t="inlineStr"/>
@@ -11104,7 +11360,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Bear-meat citatap stew with pukusakina and veggies. (party HP +600, cures freeze)</t>
+          <t>Bear citatap stew with pukusakina. (party HP +600, cures freeze)</t>
         </is>
       </c>
       <c r="E305" t="inlineStr"/>
@@ -11279,7 +11535,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Hot fried chicken. Ask before you add lemon juice. (HP +240, restores stats)</t>
+          <t>Hot fried chicken. Ask before the lemon. (HP +240, restores stats)</t>
         </is>
       </c>
       <c r="E310" t="inlineStr"/>
@@ -11420,7 +11676,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>A slightly disgusting dish made with simmered bear paw. (TP +300, cures all ailments)</t>
+          <t>Slightly disgusting simmered bear paw. (TP +300, cures all ailments)</t>
         </is>
       </c>
       <c r="E314" t="inlineStr"/>
@@ -11434,7 +11690,11 @@
           <t>A slightly disgusting dish made with simmered bear paw (+300 TP, Cure All Ailments).</t>
         </is>
       </c>
-      <c r="H314" t="inlineStr"/>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -11488,7 +11748,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Fried lamb meatballs with strong coriander scent. (TP +50, 100% evasion up)</t>
+          <t>Fried lamb meatballs. Smells of coriander. (TP +50, 100% evasion up)</t>
         </is>
       </c>
       <c r="E316" t="inlineStr"/>
@@ -11502,7 +11762,11 @@
           <t>Fried lamb meatballs with strong coriander scent (+100% EVA).</t>
         </is>
       </c>
-      <c r="H316" t="inlineStr"/>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -11522,7 +11786,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Lunch set with bird meat and bear meat mixed together. (HP +300, cures 1 ailment)</t>
+          <t>Bird meat and bear meat, mixed together. (HP +300, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E317" t="inlineStr"/>
@@ -11536,7 +11800,11 @@
           <t>Lunch set with bird meat and bear meat mixed together (+300 HP, Cure 1 Ailment).</t>
         </is>
       </c>
-      <c r="H317" t="inlineStr"/>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -11556,7 +11824,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Brave penguins gave their lives to bring you fuel and soap. (80% evasion up)</t>
+          <t>Brave penguins died to bring you fuel and soap. (80% evasion up)</t>
         </is>
       </c>
       <c r="E318" t="inlineStr"/>
@@ -11570,7 +11838,11 @@
           <t>Brave penguins gave their lives to bring you fuel and soap (+80% EVA).</t>
         </is>
       </c>
-      <c r="H318" t="inlineStr"/>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -11624,7 +11896,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Feel refreshed by the mint's cold, transcendent stimulation. (HP +200, cures sleep)</t>
+          <t>Cold, transcendent minty stimulation. (HP +200, cures sleep)</t>
         </is>
       </c>
       <c r="E320" t="inlineStr"/>
@@ -12070,7 +12342,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Sketchy in over seven ways. Get it? Like seven colors of the rainbow! (10% stun)</t>
+          <t>Sketchy in seven ways. Get it? Seven rainbow colors! (10% stun)</t>
         </is>
       </c>
       <c r="E333" t="inlineStr"/>
@@ -12084,7 +12356,11 @@
           <t>Sketchy in over seven ways. Get it? Like seven colors of the rainbow! (10% Blind).</t>
         </is>
       </c>
-      <c r="H333" t="inlineStr"/>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -12206,7 +12482,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Three aspects of the dumpling on one skewer. (party HP +180, 60% party ATK up)</t>
+          <t>Dumpling trinity on one skewer. (party HP +180, 60% party ATK up)</t>
         </is>
       </c>
       <c r="E337" t="inlineStr"/>
@@ -12316,7 +12592,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Raw meat cut fine and called a steak. Eat with caution. (HP/TP +2000, 95% 1 clone)</t>
+          <t>Raw meat called a steak. Eat with caution. (HP/TP +2000, 95% 1 clone)</t>
         </is>
       </c>
       <c r="E340" t="inlineStr"/>
@@ -12490,7 +12766,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>Glutinous steamed rice dish with big pieces of chestnut. (HP +515, 30% 1 clone)</t>
+          <t>Steamed rice with big pieces of chestnut. (HP +515, 30% 1 clone)</t>
         </is>
       </c>
       <c r="E345" t="inlineStr"/>
@@ -12504,7 +12780,11 @@
           <t>Glutinous steamed rice dish with big pieces of chestnut (+515 HP).</t>
         </is>
       </c>
-      <c r="H345" t="inlineStr"/>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -12558,7 +12838,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>Seashell-shaped snack. Sally sells them by the seashore. (HP +135, 30% accuracy up)</t>
+          <t>Sally sells these seashells by the shore. (HP +135, 30% accuracy up)</t>
         </is>
       </c>
       <c r="E347" t="inlineStr"/>
@@ -12572,7 +12852,11 @@
           <t>Seashell-shaped snack. Sally sells them by the seashore (+135 HP).</t>
         </is>
       </c>
-      <c r="H347" t="inlineStr"/>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -12592,7 +12876,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>Syrup and dry fruit. A hard candy for hard men. (party HP +165, restores stats)</t>
+          <t>A hard candy for hard men. (party HP +165, restores stats)</t>
         </is>
       </c>
       <c r="E348" t="inlineStr"/>
@@ -12631,7 +12915,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>Cake with a figurine. Whoever finds it gets to be king. (party HP +250, party TP +25)</t>
+          <t>Find the figurine, be the king. (party HP +250, party TP +25)</t>
         </is>
       </c>
       <c r="E349" t="inlineStr"/>
@@ -12670,7 +12954,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>Not everyone who eats muffins is in the mafia. The muffia? Hyuk hyuk. (HP/TP +30)</t>
+          <t>Not all who eat muffins are mafia. The muffia? Hyuk hyuk. (HP/TP +30)</t>
         </is>
       </c>
       <c r="E350" t="inlineStr"/>
@@ -12684,7 +12968,11 @@
           <t>Not everyone who eats muffins is in the mafia. The muffia? Hyuk hyuk (+30 HP/TP).</t>
         </is>
       </c>
-      <c r="H350" t="inlineStr"/>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -12704,7 +12992,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>Off the shelf or classy? Really not that different. (HP +50, 50% accuracy up)</t>
+          <t>Shelf or classy? Not that different. (HP +50, 50% accuracy up)</t>
         </is>
       </c>
       <c r="E351" t="inlineStr"/>
@@ -12742,7 +13030,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>Party pastry of fruits, custard, and jelly. (party TP +115, 70% party magic DEF up)</t>
+          <t>Fruit, custard, jelly. Party! (party TP +115, 70% party magic DEF up)</t>
         </is>
       </c>
       <c r="E352" t="inlineStr"/>
@@ -12780,7 +13068,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>A cookie cut into a simple shape. Ooh, looks like a star! (party HP +55)</t>
+          <t>A simple-shaped cookie. Ooh, looks like a star! (party HP +55)</t>
         </is>
       </c>
       <c r="E353" t="inlineStr"/>
@@ -12794,7 +13082,11 @@
           <t>A cookie cut into a simple shape. Ooh, looks like a star! (Party: +55 HP).</t>
         </is>
       </c>
-      <c r="H353" t="inlineStr"/>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -12814,7 +13106,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>A cookie cut into a somewhat complex shape. Ooh, looks like a cow! (party HP +160)</t>
+          <t>A somewhat complex cookie. Ooh, looks like a cow! (party HP +160)</t>
         </is>
       </c>
       <c r="E354" t="inlineStr"/>
@@ -12828,7 +13120,11 @@
           <t>A cookie cut into a somewhat complex shape. Ooh, looks like a cow! (Party: +160 HP).</t>
         </is>
       </c>
-      <c r="H354" t="inlineStr"/>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -12848,7 +13144,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>A cookie in a complex shape. Looks like Japan! (party HP +200, 60% party cure-all)</t>
+          <t>Cookie that looks like Japan! (party HP +200, 60% party cure-all)</t>
         </is>
       </c>
       <c r="E355" t="inlineStr"/>
@@ -12920,7 +13216,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>Rice cracker covered in plenty of cayenne powder. (HP +120, 25% Defender)</t>
+          <t>Rice cracker covered in cayenne powder. (HP +120, 25% Defender)</t>
         </is>
       </c>
       <c r="E357" t="inlineStr"/>
@@ -12934,7 +13230,11 @@
           <t>Rice cracker covered in plenty of cayenne powder (+120 HP).</t>
         </is>
       </c>
-      <c r="H357" t="inlineStr"/>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -12954,7 +13254,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>Just a cracker with tasty sauce, but dang, that's tasty. (HP +240, 50% Defender)</t>
+          <t>Just a cracker with sauce, but dang, tasty. (HP +240, 50% Defender)</t>
         </is>
       </c>
       <c r="E358" t="inlineStr"/>
@@ -12968,7 +13268,11 @@
           <t>Just a cracker with tasty sauce, but dang, that's tasty (+240 HP).</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr"/>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -13200,7 +13504,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>Colorful candy that is kneaded with two sticks. (TP +31, cures 1 ailment)</t>
+          <t>Colorful candy kneaded with two sticks. (TP +31, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E365" t="inlineStr"/>
@@ -13214,7 +13518,11 @@
           <t>Colorful candy that is kneaded with two sticks (+31 TP, Cure 1 Ailment).</t>
         </is>
       </c>
-      <c r="H365" t="inlineStr"/>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -13302,7 +13610,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Eat a long candy, live a long life. It's just math. (TP +150, 75% accuracy up)</t>
+          <t>Long candy, long life. It's just math. (TP +150, 75% accuracy up)</t>
         </is>
       </c>
       <c r="E368" t="inlineStr"/>
@@ -13316,7 +13624,11 @@
           <t>Eat a long candy, live a long life. It's just math (+150 TP).</t>
         </is>
       </c>
-      <c r="H368" t="inlineStr"/>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -13336,7 +13648,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>Rare, top-notch candy from the demon world. (party HP/TP +666, 95% party cure-all)</t>
+          <t>Top candy of the demon world. (party HP/TP +666, 95% party cure-all)</t>
         </is>
       </c>
       <c r="E369" t="inlineStr"/>
@@ -13408,7 +13720,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>Sunny-side up egg on a patty. When to break the yolk...? (HP +300, 75% ATK up)</t>
+          <t>Egg on a patty. When to break the yolk...? (HP +300, 75% ATK up)</t>
         </is>
       </c>
       <c r="E371" t="inlineStr"/>
@@ -13422,7 +13734,11 @@
           <t>Sunny-side up egg on a patty. When to break the yolk...? (+75% ATK).</t>
         </is>
       </c>
-      <c r="H371" t="inlineStr"/>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -13624,7 +13940,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>Sesame, white bean paste, and... red bean paste! (HP +400, 75% accuracy up)</t>
+          <t>Sesame, white bean and... red bean paste! (HP +400, 75% accuracy up)</t>
         </is>
       </c>
       <c r="E377" t="inlineStr"/>
@@ -13638,7 +13954,11 @@
           <t>Sesame, white bean paste, and... red bean paste! (+400 HP).</t>
         </is>
       </c>
-      <c r="H377" t="inlineStr"/>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -13692,7 +14012,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>Bright macarons with an assortment of colors. (HP +150, 75% accuracy up)</t>
+          <t>Bright macarons in assorted colors. (HP +150, 75% accuracy up)</t>
         </is>
       </c>
       <c r="E379" t="inlineStr"/>
@@ -13706,7 +14026,11 @@
           <t>Bright macarons with an assortment of colors (+150 HP).</t>
         </is>
       </c>
-      <c r="H379" t="inlineStr"/>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -13794,7 +14118,7 @@
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>Staple food on Planet Muscle. Go from ripped to jacked. (HP +300, 75% max HP up)</t>
+          <t>Planet Muscle staple. From ripped to jacked. (HP +300, 75% max HP up)</t>
         </is>
       </c>
       <c r="E382" t="inlineStr"/>
@@ -13808,7 +14132,11 @@
           <t>Staple food on Planet Muscle. Go from ripped to jacked (+300 HP).</t>
         </is>
       </c>
-      <c r="H382" t="inlineStr"/>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -13964,7 +14292,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>You know you should stop but you just can't kelp yourself. (TP +20, 40% silence)</t>
+          <t>You should stop but can't kelp yourself. (TP +20, 40% silence)</t>
         </is>
       </c>
       <c r="E387" t="inlineStr"/>
@@ -13978,7 +14306,11 @@
           <t>You know you should stop but you just can't kelp yourself (+20 TP, 40% Silence).</t>
         </is>
       </c>
-      <c r="H387" t="inlineStr"/>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -14032,7 +14364,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>Served without a warning, you're the butt of a joke. (TP +40, 60% silence)</t>
+          <t>Served unwarned, you're the butt of a joke. (TP +40, 60% silence)</t>
         </is>
       </c>
       <c r="E389" t="inlineStr"/>
@@ -14071,7 +14403,7 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>Bad looks and worse texture but weirdly addictive. (TP +50, 60% silence)</t>
+          <t>Bad looks, worse texture, weirdly addictive. (TP +50, 60% silence)</t>
         </is>
       </c>
       <c r="E390" t="inlineStr"/>
@@ -14085,7 +14417,11 @@
           <t>Bad looks and worse texture but weirdly addictive (+50 TP, 60% Silence).</t>
         </is>
       </c>
-      <c r="H390" t="inlineStr"/>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -14105,7 +14441,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>A flattened octopus. Plenty to go around. (party HP +160, 20% party magic DEF up)</t>
+          <t>Flat octopus. Plenty for all. (party HP +160, 20% party magic DEF up)</t>
         </is>
       </c>
       <c r="E391" t="inlineStr"/>
@@ -14212,7 +14548,7 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>Apparently the primary source of sustenance for one particular race. (HP/TP +200)</t>
+          <t>The main sustenance of one particular race. (HP/TP +200)</t>
         </is>
       </c>
       <c r="E394" t="inlineStr"/>
@@ -14226,7 +14562,11 @@
           <t>Apparently the primary source of sustenance for one particular race (+200 HP/TP).</t>
         </is>
       </c>
-      <c r="H394" t="inlineStr"/>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -14280,7 +14620,7 @@
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>Tastes... sweet. Nothing but sweet. Not to be confused with balaclava. (TP +44)</t>
+          <t>Nothing but sweet. Not to be confused with balaclava. (TP +44)</t>
         </is>
       </c>
       <c r="E396" t="inlineStr"/>
@@ -14294,7 +14634,11 @@
           <t>Tastes... sweet. Nothing but sweet. Not to be confused with balaclava (+44 TP).</t>
         </is>
       </c>
-      <c r="H396" t="inlineStr"/>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -14314,7 +14658,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>A runny, sugary snack. The calorie content must be through the roof. (TP +72)</t>
+          <t>A runny, sugary snack. Calories through the roof. (TP +72)</t>
         </is>
       </c>
       <c r="E397" t="inlineStr"/>
@@ -14328,7 +14672,11 @@
           <t>A runny, sugary snack. The calorie content must be through the roof (+72 TP).</t>
         </is>
       </c>
-      <c r="H397" t="inlineStr"/>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -14450,7 +14798,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>Waffle made with rice flour. Comes out mochi-ish. (TP +50, restores stats)</t>
+          <t>Rice flour waffle. Comes out mochi-ish. (TP +50, restores stats)</t>
         </is>
       </c>
       <c r="E401" t="inlineStr"/>
@@ -14464,7 +14812,11 @@
           <t>Waffle made with rice flour. Comes out mochi-ish (+50 TP, Clear Debuffs).</t>
         </is>
       </c>
-      <c r="H401" t="inlineStr"/>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -14484,7 +14836,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>A sweet waffle with syrup mixed into the batter. (TP +85, cures all ailments)</t>
+          <t>Sweet waffle with syrup in the batter. (TP +85, cures all ailments)</t>
         </is>
       </c>
       <c r="E402" t="inlineStr"/>
@@ -14498,7 +14850,11 @@
           <t>A sweet waffle with syrup mixed into the batter (+85 TP, Cure All Ailments).</t>
         </is>
       </c>
-      <c r="H402" t="inlineStr"/>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -14518,7 +14874,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>Luxury pancakes like you only get at overpriced hotels. (TP +160, cures all ailments)</t>
+          <t>Overpriced-hotel luxury pancakes. (TP +160, cures all ailments)</t>
         </is>
       </c>
       <c r="E403" t="inlineStr"/>
@@ -14532,7 +14888,11 @@
           <t>Luxury pancakes like you only get at overpriced hotels (+160 TP, Cure All Ailments).</t>
         </is>
       </c>
-      <c r="H403" t="inlineStr"/>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -14552,7 +14912,7 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>Which end do you eat it from? It's a matter of scholarly debate. (TP +30)</t>
+          <t>Which end to eat first? A matter of scholarly debate. (TP +30)</t>
         </is>
       </c>
       <c r="E404" t="inlineStr"/>
@@ -14566,7 +14926,11 @@
           <t>Which end do you eat it from? It's a matter of scholarly debate (+30 TP).</t>
         </is>
       </c>
-      <c r="H404" t="inlineStr"/>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -14586,7 +14950,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>Tough rye bread that poses a challenge for seniors with weak teeth. (HP +58)</t>
+          <t>Tough rye bread. A challenge for weak teeth. (HP +58)</t>
         </is>
       </c>
       <c r="E405" t="inlineStr"/>
@@ -14600,7 +14964,11 @@
           <t>Tough rye bread that poses a challenge for seniors with weak teeth (+58 HP).</t>
         </is>
       </c>
-      <c r="H405" t="inlineStr"/>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -14620,7 +14988,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>Red bean bun of fine gold wheat. Diabetics should avoid it. (HP +400, 80% Defender)</t>
+          <t>Fine gold wheat bun. Diabetics, avoid it. (HP +400, 80% Defender)</t>
         </is>
       </c>
       <c r="E406" t="inlineStr"/>
@@ -14798,7 +15166,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>Invokes the undeniable urge to rap. You'll be a real Kandy-e West. (HP +70)</t>
+          <t>Brings the urge to rap. You'll be a real Kandy-e West. (HP +70)</t>
         </is>
       </c>
       <c r="E411" t="inlineStr"/>
@@ -14812,7 +15180,11 @@
           <t>Invokes the undeniable urge to rap. You'll be a real Kandy-e West (+70 HP).</t>
         </is>
       </c>
-      <c r="H411" t="inlineStr"/>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -14832,7 +15204,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>A high-class rusk coated in white chocolate. Mindblowingly delicious. (HP +150)</t>
+          <t>High-class white chocolate rusk. Mindblowingly delicious. (HP +150)</t>
         </is>
       </c>
       <c r="E412" t="inlineStr"/>
@@ -14846,7 +15218,11 @@
           <t>A high-class rusk coated in white chocolate. Mindblowingly delicious (+150 HP).</t>
         </is>
       </c>
-      <c r="H412" t="inlineStr"/>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -14866,7 +15242,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>A candy so sweet it will cause your brain to melt. (HP +300, 30% silence)</t>
+          <t>Candy so sweet your brain will melt. (HP +300, 30% silence)</t>
         </is>
       </c>
       <c r="E413" t="inlineStr"/>
@@ -14880,7 +15256,11 @@
           <t>A candy so sweet it will cause your brain to melt (+300 HP, 30% Silence).</t>
         </is>
       </c>
-      <c r="H413" t="inlineStr"/>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -14934,7 +15314,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>Eat it and you'll sweat from every orifice you've got. (HP +50, cures freeze)</t>
+          <t>You'll sweat from every orifice you've got. (HP +50, cures freeze)</t>
         </is>
       </c>
       <c r="E415" t="inlineStr"/>
@@ -14948,7 +15328,11 @@
           <t>Eat it and you'll sweat from every orifice you've got (+50 HP, Cure Freeze).</t>
         </is>
       </c>
-      <c r="H415" t="inlineStr"/>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -14968,7 +15352,7 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>First-timers will lose consciousness due to the spice. (HP/TP +75, 15% paralysis)</t>
+          <t>First-timers pass out from the spice. (HP/TP +75, 15% paralysis)</t>
         </is>
       </c>
       <c r="E416" t="inlineStr"/>
@@ -14982,7 +15366,11 @@
           <t>First-timers will lose consciousness due to the spice (+75 HP/TP, 15% Paralysis).</t>
         </is>
       </c>
-      <c r="H416" t="inlineStr"/>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -15002,7 +15390,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>So spicy it's out of this world. One call and they deliver. (HP +400, 80% silence)</t>
+          <t>Out-of-this-world spicy. They deliver. (HP +400, 80% silence)</t>
         </is>
       </c>
       <c r="E417" t="inlineStr"/>
@@ -15075,7 +15463,7 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Donut with red bean paste on the inside, sugar coating on the outside. (HP +200)</t>
+          <t>Donut with red bean paste inside, sugar coating outside. (HP +200)</t>
         </is>
       </c>
       <c r="E419" t="inlineStr"/>
@@ -15089,7 +15477,11 @@
           <t>Donut with red bean paste on the inside, sugar coating on the outside (+200 HP).</t>
         </is>
       </c>
-      <c r="H419" t="inlineStr"/>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -15215,7 +15607,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Taiyaki with matcha mixed into the batter. Looks a little gross. (HP +200, TP +40)</t>
+          <t>Matcha in the batter. Looks a little gross. (HP +200, TP +40)</t>
         </is>
       </c>
       <c r="E423" t="inlineStr"/>
@@ -15229,7 +15621,11 @@
           <t>Taiyaki with matcha mixed into the batter. Looks a little gross (+200 HP, +40 TP).</t>
         </is>
       </c>
-      <c r="H423" t="inlineStr"/>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -15249,7 +15645,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>The shrooms of the hills despise the coddled city bamboo shoots. (TP +40)</t>
+          <t>Hill shrooms despise the coddled city bamboo shoots. (TP +40)</t>
         </is>
       </c>
       <c r="E424" t="inlineStr"/>
@@ -15263,7 +15659,11 @@
           <t>The shrooms of the hills despise the coddled city bamboo shoots (+40 TP).</t>
         </is>
       </c>
-      <c r="H424" t="inlineStr"/>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -15317,7 +15717,7 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>The mushroom formerly known as matsutake. They're... fine. (25% Divine Shield)</t>
+          <t>Formerly known as matsutake. They're... fine. (25% Divine Shield)</t>
         </is>
       </c>
       <c r="E426" t="inlineStr"/>
@@ -15331,7 +15731,11 @@
           <t>The mushroom formerly known as matsutake. They're... fine.</t>
         </is>
       </c>
-      <c r="H426" t="inlineStr"/>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -15351,7 +15755,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Yellow with red spots. Eat it, and you might get bigger. (50% max HP up)</t>
+          <t>Yellow with red spots. Eat it and you may grow. (50% max HP up)</t>
         </is>
       </c>
       <c r="E427" t="inlineStr"/>
@@ -15365,7 +15769,11 @@
           <t>Yellow with red spots. Eat it, and you might get bigger.</t>
         </is>
       </c>
-      <c r="H427" t="inlineStr"/>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -15589,7 +15997,7 @@
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Opulent Chinese vegetable dish. Contains no meat. For some reason. (TP +150)</t>
+          <t>Opulent vegetable dish. No meat. For some reason. (TP +150)</t>
         </is>
       </c>
       <c r="E434" t="inlineStr"/>
@@ -15603,7 +16011,11 @@
           <t>Opulent Chinese vegetable dish. Contains no meat. For some reason (+150 TP).</t>
         </is>
       </c>
-      <c r="H434" t="inlineStr"/>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -15623,7 +16035,7 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Sticky pudding with raisins. Just pudding. Honestly. (HP +100, cures 1 ailment)</t>
+          <t>Just raisin pudding. Honestly. (HP +100, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E435" t="inlineStr"/>
@@ -15662,7 +16074,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>A cakey treat filled with delicious red bean paste. (HP +280, cures 1 ailment)</t>
+          <t>Cakey treat filled with red bean paste. (HP +280, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E436" t="inlineStr"/>
@@ -15676,7 +16088,11 @@
           <t>A cakey treat filled with delicious red bean paste (+280 HP, Cure 1 Ailment).</t>
         </is>
       </c>
-      <c r="H436" t="inlineStr"/>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -15696,7 +16112,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Ol' reliable. You can't go wrong with bean paste. (TP +125, 65% Insurance)</t>
+          <t>Ol' reliable. Bean paste can't go wrong. (TP +125, 65% Insurance)</t>
         </is>
       </c>
       <c r="E437" t="inlineStr"/>
@@ -15710,7 +16126,11 @@
           <t>Ol' reliable. You can't go wrong with bean paste (+125 TP).</t>
         </is>
       </c>
-      <c r="H437" t="inlineStr"/>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -15730,7 +16150,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Soup made of leftovers. Liver and let die! (party TP +10, 20% party cure-all)</t>
+          <t>Leftovers. Liver and let die! (party TP +10, 20% party cure-all)</t>
         </is>
       </c>
       <c r="E438" t="inlineStr"/>
@@ -15768,7 +16188,7 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>The unagi's not always good, but the sauce is. (party TP +25, 40% party cure-all)</t>
+          <t>Come for the sauce, not the eel. (party TP +25, 40% party cure-all)</t>
         </is>
       </c>
       <c r="E439" t="inlineStr"/>
@@ -15806,7 +16226,7 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Dead eels on rice. You wouldn't want any. (party TP +50, 60% party cure-all)</t>
+          <t>Dead eels on rice. You'd pass. (party TP +50, 60% party cure-all)</t>
         </is>
       </c>
       <c r="E440" t="inlineStr"/>
@@ -15844,7 +16264,7 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Sushi roll of sticky, smelly, fermented soybeans. Yum...? (HP/TP +30, 50% silence)</t>
+          <t>Sticky, smelly soybean sushi. Yum...? (HP/TP +30, 50% silence)</t>
         </is>
       </c>
       <c r="E441" t="inlineStr"/>
@@ -15883,7 +16303,7 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>You must be mindful of your surroundings when eating this. (HP/TP +60, 60% silence)</t>
+          <t>Mind your surroundings when eating this. (HP/TP +60, 60% silence)</t>
         </is>
       </c>
       <c r="E442" t="inlineStr"/>
@@ -15897,7 +16317,11 @@
           <t>You must be mindful of your surroundings when eating this (+60 HP/TP, 60% Silence).</t>
         </is>
       </c>
-      <c r="H442" t="inlineStr"/>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -15985,7 +16409,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>Somewhat grotesque when the fish has the face of a man. (HP +100, 40% stun)</t>
+          <t>Grotesque when the fish has a man's face. (HP +100, 40% stun)</t>
         </is>
       </c>
       <c r="E445" t="inlineStr"/>
@@ -15999,7 +16423,11 @@
           <t>Somewhat grotesque when the fish has the face of a man (+100 HP, 40% Blind).</t>
         </is>
       </c>
-      <c r="H445" t="inlineStr"/>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -16053,7 +16481,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Bonito so dry it's a blunt weapon. The world's hardest food. (HP +200, 80% DEF up)</t>
+          <t>Bonito so dry it's a blunt weapon. (HP +200, 80% DEF up)</t>
         </is>
       </c>
       <c r="E447" t="inlineStr"/>
@@ -16067,7 +16495,11 @@
           <t>Bonito so dry it's a blunt weapon. The world's hardest food (+80% DEF).</t>
         </is>
       </c>
-      <c r="H447" t="inlineStr"/>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -16121,7 +16553,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>A simple but deep sushi. Make this your last order to look cultured. (HP +50, TP +10)</t>
+          <t>Simple but deep. Order it last to look cultured. (HP +50, TP +10)</t>
         </is>
       </c>
       <c r="E449" t="inlineStr"/>
@@ -16135,7 +16567,11 @@
           <t>A simple but deep sushi. Make this your last order to look cultured (+50 HP, +10 TP).</t>
         </is>
       </c>
-      <c r="H449" t="inlineStr"/>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -16155,7 +16591,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Bitter jelly good for the skin. Not so great for the tortoise. (cures all ailments)</t>
+          <t>Good for the skin. Not so for the tortoise. (cures all ailments)</t>
         </is>
       </c>
       <c r="E450" t="inlineStr"/>
@@ -16194,7 +16630,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Genuine, real turtle soup! Would I lie to you? (cures all ailments, 40% max HP up)</t>
+          <t>Real turtle! Would I lie to you? (cures all ailments, 40% max HP up)</t>
         </is>
       </c>
       <c r="E451" t="inlineStr"/>
@@ -16232,7 +16668,7 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>Made in an earthenware pot. Delicious but steep. (cures all ailments, TP +125)</t>
+          <t>Earthenware pot. Delicious but steep. (cures all ailments, TP +125)</t>
         </is>
       </c>
       <c r="E452" t="inlineStr"/>
@@ -16305,7 +16741,7 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>Bento with only meat and rice. Get those veggies out of here! (HP +150, 50% ATK up)</t>
+          <t>Only meat and rice. Veggies, get out of here! (HP +150, 50% ATK up)</t>
         </is>
       </c>
       <c r="E454" t="inlineStr"/>
@@ -16319,7 +16755,11 @@
           <t>Bento with only meat and rice. Get those veggies out of here! (+50% ATK).</t>
         </is>
       </c>
-      <c r="H454" t="inlineStr"/>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -16339,7 +16779,7 @@
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>Sukiyaki bento with super luxurious wagyu included. (HP +200, 70% ATK up)</t>
+          <t>Sukiyaki bento with super luxurious wagyu. (HP +200, 70% ATK up)</t>
         </is>
       </c>
       <c r="E455" t="inlineStr"/>
@@ -16353,7 +16793,11 @@
           <t>Sukiyaki bento with super luxurious wagyu included (+70% ATK).</t>
         </is>
       </c>
-      <c r="H455" t="inlineStr"/>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -16475,7 +16919,7 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>Try to point out that it's yellow, and a rep will appear to call it gold. (TP +60)</t>
+          <t>Call it yellow and a rep will appear to call it gold. (TP +60)</t>
         </is>
       </c>
       <c r="E459" t="inlineStr"/>
@@ -16489,7 +16933,11 @@
           <t>Try to point out that it's yellow, and a rep will appear to call it gold (+60 TP).</t>
         </is>
       </c>
-      <c r="H459" t="inlineStr"/>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -16509,7 +16957,7 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>Don't drink too much if you like your brain cells. (TP +75, 20% instakill)</t>
+          <t>Go easy if you like your brain cells. (TP +75, 20% instakill)</t>
         </is>
       </c>
       <c r="E460" t="inlineStr"/>
@@ -16523,7 +16971,11 @@
           <t>Don't drink too much if you like your brain cells (+75 TP).</t>
         </is>
       </c>
-      <c r="H460" t="inlineStr"/>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -16577,7 +17029,7 @@
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>Cheap and delicious. Sometimes filled with pudding. (HP +135, cancels Shadow Sew)</t>
+          <t>Cheap, tasty. Sometimes has pudding. (HP +135, cancels Shadow Sew)</t>
         </is>
       </c>
       <c r="E462" t="inlineStr"/>
@@ -16616,7 +17068,7 @@
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>Mochi with mugwort. You can never have too much mugwort! (HP +225, cures 1 ailment)</t>
+          <t>You can never have too much mugwort! (HP +225, cures 1 ailment)</t>
         </is>
       </c>
       <c r="E463" t="inlineStr"/>
@@ -16630,7 +17082,11 @@
           <t>Mochi with mugwort. You can never have too much mugwort! (+225 HP, Cure 1 Ailment).</t>
         </is>
       </c>
-      <c r="H463" t="inlineStr"/>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -16752,7 +17208,7 @@
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>Handle it with care, or the cream will spurt all over you. (HP +200, 25% DEF up)</t>
+          <t>Careful, or the cream will spurt all over you. (HP +200, 25% DEF up)</t>
         </is>
       </c>
       <c r="E467" t="inlineStr"/>
@@ -16824,7 +17280,7 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>Triple-stack of pancakes in sticky maple syrup. (party HP +180, 25% party ATK up)</t>
+          <t>Triple-stack in maple syrup. (party HP +180, 25% party ATK up)</t>
         </is>
       </c>
       <c r="E469" t="inlineStr"/>
@@ -16862,7 +17318,7 @@
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>It means white mountain. And yet, yellow cake. Y u do dis? (HP +300, 25% accuracy up)</t>
+          <t>White mountain, yellow cake. Y u do dis? (HP +300, 25% accuracy up)</t>
         </is>
       </c>
       <c r="E470" t="inlineStr"/>
@@ -16876,7 +17332,11 @@
           <t>It means white mountain. And yet, yellow cake. Y u do dis? (+300 HP).</t>
         </is>
       </c>
-      <c r="H470" t="inlineStr"/>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -16930,7 +17390,7 @@
       </c>
       <c r="D472" t="inlineStr">
         <is>
-          <t>A multi-layered, doughy pie cake. (party HP +300, 25% party magic DEF up)</t>
+          <t>Multi-layered doughy pie cake. (party HP +300, 25% party magic DEF up)</t>
         </is>
       </c>
       <c r="E472" t="inlineStr"/>
@@ -16944,7 +17404,11 @@
           <t>A multi-layered, doughy pie cake (Party: +300 HP).</t>
         </is>
       </c>
-      <c r="H472" t="inlineStr"/>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -16964,7 +17428,7 @@
       </c>
       <c r="D473" t="inlineStr">
         <is>
-          <t>A luxury item perfect for souvenirs or gifts. (party TP +200, 40% party DEF up)</t>
+          <t>A luxury souvenir or gift. (party TP +200, 40% party DEF up)</t>
         </is>
       </c>
       <c r="E473" t="inlineStr"/>
@@ -17002,7 +17466,7 @@
       </c>
       <c r="D474" t="inlineStr">
         <is>
-          <t>Maple leaf-shaped souvenir confection. Even better as ice cream. (HP +60, TP +15)</t>
+          <t>Maple leaf souvenir. Even better as ice cream. (HP +60, TP +15)</t>
         </is>
       </c>
       <c r="E474" t="inlineStr"/>
@@ -17016,7 +17480,11 @@
           <t>Maple leaf-shaped souvenir confection. Even better as ice cream (+60 HP, +15 TP).</t>
         </is>
       </c>
-      <c r="H474" t="inlineStr"/>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -17036,7 +17504,7 @@
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>Liquor brewed from millet. Its mature flavor can become a habit. (HP +125, 40% sleep)</t>
+          <t>Millet liquor. Its mature flavor can be a habit. (HP +125, 40% sleep)</t>
         </is>
       </c>
       <c r="E475" t="inlineStr"/>
@@ -17050,7 +17518,11 @@
           <t>Liquor brewed from millet. Its mature flavor can become a habit (+125 HP, 40% Sleep).</t>
         </is>
       </c>
-      <c r="H475" t="inlineStr"/>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -17070,7 +17542,7 @@
       </c>
       <c r="D476" t="inlineStr">
         <is>
-          <t>Its mascot creature has yet to be identified by science. (HP +165, 20% stun)</t>
+          <t>Its mascot is still unidentified by science. (HP +165, 20% stun)</t>
         </is>
       </c>
       <c r="E476" t="inlineStr"/>
@@ -17109,7 +17581,7 @@
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>Canned whale. Slowly vanishing from shelves. (HP +200, 25% Divine Shield)</t>
+          <t>Canned whale. Vanishing from shelves. (HP +200, 25% Divine Shield)</t>
         </is>
       </c>
       <c r="E477" t="inlineStr"/>
@@ -17123,7 +17595,11 @@
           <t>Canned whale. Slowly vanishing from shelves (+200 HP).</t>
         </is>
       </c>
-      <c r="H477" t="inlineStr"/>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -17351,7 +17827,7 @@
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>Made from only the gloopiest cuts of the slime. (30 fixed damage, 5% slow)</t>
+          <t>Only the gloopiest cuts of slime. (30 fixed damage, 5% slow)</t>
         </is>
       </c>
       <c r="E484" t="inlineStr"/>
@@ -17365,7 +17841,11 @@
           <t>Made from only the gloopiest cuts of the slime (Speed DOWN -10%.).</t>
         </is>
       </c>
-      <c r="H484" t="inlineStr"/>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -17419,7 +17899,7 @@
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>Bavarian cream full of slime. Appetizing? (party 50 fixed damage, 75% strips buffs)</t>
+          <t>Full of slime. Appetizing? (party 50 fixed damage, 75% strips buffs)</t>
         </is>
       </c>
       <c r="E486" t="inlineStr"/>
@@ -17457,7 +17937,7 @@
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>Spray that turns you into a super sadist for a few minutes. (50% Berserk)</t>
+          <t>Spray that makes you a super sadist for a few minutes. (50% Berserk)</t>
         </is>
       </c>
       <c r="E487" t="inlineStr"/>
@@ -17471,7 +17951,11 @@
           <t>Spray that turns you into a super sadist for a few minutes (+50% ATK).</t>
         </is>
       </c>
-      <c r="H487" t="inlineStr"/>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -17491,7 +17975,7 @@
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>Feeling foreign. You're a stranger in a strange land. (75% Berserk, 75% stun)</t>
+          <t>You're a stranger in a strange land. (75% Berserk, 75% stun)</t>
         </is>
       </c>
       <c r="E488" t="inlineStr"/>
@@ -17529,7 +18013,7 @@
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>Canned dragon meat. Rare, expensive, a little smelly. (TP +150, cures all ailments)</t>
+          <t>Rare, pricey, slightly smelly meat. (TP +150, cures all ailments)</t>
         </is>
       </c>
       <c r="E489" t="inlineStr"/>
@@ -17602,7 +18086,7 @@
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>Some never tried this sake, but none tried it only once. (HP +150, 15% sleep)</t>
+          <t>Some never tried it, none tried it only once. (HP +150, 15% sleep)</t>
         </is>
       </c>
       <c r="E491" t="inlineStr"/>
@@ -17641,7 +18125,7 @@
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>Sake that intoxicates even heavy drinkers. Super harsh. (HP +300, 20% stun)</t>
+          <t>Intoxicates even heavy drinkers. Super harsh. (HP +300, 20% stun)</t>
         </is>
       </c>
       <c r="E492" t="inlineStr"/>
@@ -17680,7 +18164,7 @@
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>Port wine carefully aged for over a hundred years. (HP +400, 20% sleep)</t>
+          <t>Port wine aged for over a hundred years. (HP +400, 20% sleep)</t>
         </is>
       </c>
       <c r="E493" t="inlineStr"/>
@@ -17694,7 +18178,11 @@
           <t>Port wine carefully aged for over a hundred years (+400 HP, 20% Sleep).</t>
         </is>
       </c>
-      <c r="H493" t="inlineStr"/>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -17782,7 +18270,7 @@
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>Dish made by shoving waterfowls into a dragon corpse. (HP/TP +200, 50% paralysis)</t>
+          <t>Waterfowl shoved into a dragon corpse. (HP/TP +200, 50% paralysis)</t>
         </is>
       </c>
       <c r="E496" t="inlineStr"/>
@@ -17796,7 +18284,11 @@
           <t>Dish made by shoving waterfowls into a dragon corpse (+200 HP/TP, 50% Paralysis).</t>
         </is>
       </c>
-      <c r="H496" t="inlineStr"/>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -17850,7 +18342,7 @@
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>A snack so hard, you might chip a tooth when you bite into it. (HP +200, TP +50)</t>
+          <t>So hard, a bite might chip your tooth. (HP +200, TP +50)</t>
         </is>
       </c>
       <c r="E498" t="inlineStr"/>
@@ -17864,7 +18356,11 @@
           <t>A snack so hard, you might chip a tooth when you bite into it (+200 HP, +50 TP).</t>
         </is>
       </c>
-      <c r="H498" t="inlineStr"/>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -17952,7 +18448,7 @@
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>Meat is most delicious when it's almost rotten... or so they say. (35% poison)</t>
+          <t>Meat is best when almost rotten... or so they say. (35% poison)</t>
         </is>
       </c>
       <c r="E501" t="inlineStr"/>
@@ -17966,7 +18462,11 @@
           <t>Meat is most delicious when it's almost rotten... or so they say (70% Poison).</t>
         </is>
       </c>
-      <c r="H501" t="inlineStr"/>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
@@ -17986,7 +18486,7 @@
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>Meat that shines suspiciously. Steroids in meat form. (50% poison, 40% paralysis)</t>
+          <t>Shines suspiciously. Steroids as meat. (50% poison, 40% paralysis)</t>
         </is>
       </c>
       <c r="E502" t="inlineStr"/>
@@ -18229,7 +18729,7 @@
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>Beverage squeezed out of an apple creature's insides. (HP/TP +100, 40% poison)</t>
+          <t>Squeezed from an apple creature's guts. (HP/TP +100, 40% poison)</t>
         </is>
       </c>
       <c r="E509" t="inlineStr"/>
@@ -18243,7 +18743,11 @@
           <t>Beverage squeezed out of an apple creature's insides (+100 HP/TP, 40% Poison).</t>
         </is>
       </c>
-      <c r="H509" t="inlineStr"/>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
@@ -18297,7 +18801,7 @@
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>Beverage squeezed out of a melon creature's insides. (HP/TP +100, 90% paralysis)</t>
+          <t>Squeezed from a melon creature's guts. (HP/TP +100, 90% paralysis)</t>
         </is>
       </c>
       <c r="E511" t="inlineStr"/>
@@ -18311,7 +18815,11 @@
           <t>Beverage squeezed out of a melon creature's insides (+100 HP/TP, 90% Paralysis).</t>
         </is>
       </c>
-      <c r="H511" t="inlineStr"/>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
@@ -18331,7 +18839,7 @@
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>Unrelated to the anime girl whose face gets eaten. (HP/TP +200, 80% paralysis)</t>
+          <t>Not the anime girl whose face gets eaten. (HP/TP +200, 80% paralysis)</t>
         </is>
       </c>
       <c r="E512" t="inlineStr"/>
@@ -18370,7 +18878,7 @@
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>Beverage squeezed out of a banana creature's insides. (HP/TP +100, 40% silence)</t>
+          <t>Squeezed from a banana creature's guts. (HP/TP +100, 40% silence)</t>
         </is>
       </c>
       <c r="E513" t="inlineStr"/>
@@ -18384,7 +18892,11 @@
           <t>Beverage squeezed out of a banana creature's insides (+100 HP/TP, 40% Silence).</t>
         </is>
       </c>
-      <c r="H513" t="inlineStr"/>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
@@ -18506,7 +19018,7 @@
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>Can be used as herbal medicine. It has a strong scent. (cures all ailments)</t>
+          <t>Herbal medicine with a strong scent. (cures all ailments)</t>
         </is>
       </c>
       <c r="E517" t="inlineStr"/>
@@ -18520,7 +19032,11 @@
           <t>Can be used as herbal medicine. It has a strong scent (Cure All Ailments).</t>
         </is>
       </c>
-      <c r="H517" t="inlineStr"/>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
@@ -18540,7 +19056,7 @@
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>A mandra trefoil, used as a graduation charm. (party TP +150, 60% party magic DEF up)</t>
+          <t>A mandra graduation charm. (party TP +150, 60% party magic DEF up)</t>
         </is>
       </c>
       <c r="E518" t="inlineStr"/>
@@ -18714,7 +19230,7 @@
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>Too much of it will cause severe hallucinations. Not the good kind. (80% Defender)</t>
+          <t>Too much causes hallucinations. Not the good kind. (80% Defender)</t>
         </is>
       </c>
       <c r="E523" t="inlineStr"/>
@@ -18728,7 +19244,11 @@
           <t>Too much of it will cause severe hallucinations. Not the good kind.</t>
         </is>
       </c>
-      <c r="H523" t="inlineStr"/>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
@@ -18748,7 +19268,7 @@
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>Fresh-squeezed mandra juice. Nice and pulpy. (party HP/TP +2000, 90% party cure-all)</t>
+          <t>Fresh-squeezed and pulpy. (party HP/TP +2000, 90% party cure-all)</t>
         </is>
       </c>
       <c r="E524" t="inlineStr"/>
@@ -18786,7 +19306,7 @@
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>Said to bring good fortune. Does anyone actually believe that? (party HP/TP +1000)</t>
+          <t>Said to bring luck. Does anyone believe that? (party HP/TP +1000)</t>
         </is>
       </c>
       <c r="E525" t="inlineStr"/>
@@ -18800,7 +19320,11 @@
           <t>Said to bring good fortune. Does anyone actually believe that? (Party: +1000 HP/TP).</t>
         </is>
       </c>
-      <c r="H525" t="inlineStr"/>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
@@ -18990,7 +19514,7 @@
       </c>
       <c r="D531" t="inlineStr">
         <is>
-          <t>Made to achieve sake supremacy. To sake-cceed. (HP/TP +50, cures all ailments)</t>
+          <t>For sake supremacy. To sake-cceed. (HP/TP +50, cures all ailments)</t>
         </is>
       </c>
       <c r="E531" t="inlineStr"/>
@@ -19029,7 +19553,7 @@
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>Denizens of the world above say these pair well with tea. (TP +1000, 90% Insurance)</t>
+          <t>Heaven's denizens pair these with tea. (TP +1000, 90% Insurance)</t>
         </is>
       </c>
       <c r="E532" t="inlineStr"/>
@@ -19101,7 +19625,7 @@
       </c>
       <c r="D534" t="inlineStr">
         <is>
-          <t>Rice cake that crumbles from the outside as you eat it. (TP +130, 75% Divine Shield)</t>
+          <t>Rice cake that crumbles as you eat it. (TP +130, 75% Divine Shield)</t>
         </is>
       </c>
       <c r="E534" t="inlineStr"/>
@@ -19115,7 +19639,11 @@
           <t>Rice cake that crumbles from the outside as you eat it (+130 TP).</t>
         </is>
       </c>
-      <c r="H534" t="inlineStr"/>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -19135,7 +19663,7 @@
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>Sweet-smelling beverage of liquified mana crystals. (TP +999, cures all ailments)</t>
+          <t>Sweet drink of liquified mana crystals. (TP +999, cures all ailments)</t>
         </is>
       </c>
       <c r="E535" t="inlineStr"/>
@@ -19174,7 +19702,7 @@
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>Drink that lights a fire in your loins. Yowch! Hot! (HP +5000, 99% max HP up)</t>
+          <t>Lights a fire in your loins. Yowch! Hot! (HP +5000, 99% max HP up)</t>
         </is>
       </c>
       <c r="E536" t="inlineStr"/>
@@ -19246,7 +19774,7 @@
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>The most treasured treasure of the Dragon Palace... cures Freeze. (cures freeze)</t>
+          <t>The Dragon Palace's most treasured treasure... (cures freeze)</t>
         </is>
       </c>
       <c r="E538" t="inlineStr"/>
@@ -19260,7 +19788,11 @@
           <t>The most treasured treasure of the Dragon Palace... cures Freeze (Cure Freeze).</t>
         </is>
       </c>
-      <c r="H538" t="inlineStr"/>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -19280,7 +19812,7 @@
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>Tender green bud held by the former ruler of the world. (95% strips buffs)</t>
+          <t>Green bud held by the former ruler of the world. (95% strips buffs)</t>
         </is>
       </c>
       <c r="E539" t="inlineStr"/>
@@ -19294,7 +19826,11 @@
           <t>Tender green bud held by the former ruler of the world.</t>
         </is>
       </c>
-      <c r="H539" t="inlineStr"/>
+      <c r="H539" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -19314,7 +19850,7 @@
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>A magical egg. There's a whole new world inside it. (HP +1000, restores stats)</t>
+          <t>There's a whole new world inside it. (HP +1000, restores stats)</t>
         </is>
       </c>
       <c r="E540" t="inlineStr"/>
@@ -19328,7 +19864,11 @@
           <t>A magical egg. There's a whole new world inside it (+1000 HP, Clear Debuffs).</t>
         </is>
       </c>
-      <c r="H540" t="inlineStr"/>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -19348,7 +19888,7 @@
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>Proof that you've attended all of Miss Euthys's lectures. (leaves the dungeon)</t>
+          <t>Proof you attended all of Miss Euthys's lectures. (leaves the dungeon)</t>
         </is>
       </c>
       <c r="E541" t="inlineStr"/>
@@ -19362,7 +19902,11 @@
           <t>Proof that you've attended all of Miss Euthys's lectures (Escape Dungeon).</t>
         </is>
       </c>
-      <c r="H541" t="inlineStr"/>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>original sentence shortened to fit</t>
+        </is>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -20608,7 +21152,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>QoL_Desc is the text the build writes into ItemData.pck. One line, 85 characters at most.</t>
+          <t>QoL_Desc is the text the build writes into ItemData.pck. One line, 70 characters at most (the battle bar).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: close the QoL roadmap
close the QoL roadmap: more item effects, Provoke enmity, player
package, final docs

34 more items state what they do (spell items, speed up, Whale Soup,
Cloaking Device), decoded with the DT2-2 wiki's item list. Provoke and
Attract show the enmity they draw. package_variant.py zips the variant
with originals to uninstall and a player README. The roadmap lists what
is done, what the project must review and what is blocked.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_item_text.xlsx
+++ b/mod_project/data_tables/qol_item_text.xlsx
@@ -1861,7 +1861,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>A Souffle special. Makes a mysterious ticking noise.</t>
+          <t>A Souffle special. Makes a mysterious ticking noise. (Fire Blast Lv10)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -1875,11 +1875,7 @@
           <t>A Souffle special. Makes a mysterious ticking noise (10 Fixed Dmg).</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2264,7 +2260,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>The cage of a flame beast that's too hot to handle.</t>
+          <t>The cage of a flame beast that's too hot to handle. (Fire Blast Lv1)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2278,11 +2274,7 @@
           <t>The cage of a flame beast that's too hot to handle.</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2302,7 +2294,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>A book chock-full of information about demons.</t>
+          <t>A book chock-full of information about demons. (Soul Absorb Lv2)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -2316,11 +2308,7 @@
           <t>A book chock-full of information about demons.</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3294,7 +3282,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Compendium of every style made by a master fistfighter.</t>
+          <t>Every style of a master fistfighter. (85% Berserk, 85% speed up)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -3310,7 +3298,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3643,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>A stick for kids. To play with. Get your mind out of the gutter.</t>
+          <t>A kids' toy stick. Get your mind out of the gutter. (Soul Absorb Lv6)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3671,7 +3659,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3715,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>The handle of a toilet plunger.</t>
+          <t>The handle of a toilet plunger. (Ice Edge Lv2)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -3741,11 +3729,7 @@
           <t>The handle of a toilet plunger.</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4020,7 +4004,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>A glass bottle containing pure electricity. Shocking!</t>
+          <t>A glass bottle of pure electricity. Shocking! (Thunder Chain Lv2)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -4036,7 +4020,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4187,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Creepy black fire. It was always burning since the world's been turning.</t>
+          <t>Creepy black fire, burning since the world's turning. (Fire Blast Lv2)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -4219,7 +4203,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4645,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Apparently a product of lunar metallurgy. Who can say?</t>
+          <t>Apparently a product of lunar metallurgy. Who can say? (Meteor Lv1)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4675,11 +4659,7 @@
           <t>Apparently a product of lunar metallurgy. Who can say?</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4767,7 +4747,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>It's better not to make contracts with your soul. Even with other humans.</t>
+          <t>No contracts with your soul. Even with other humans. (Soul Absorb Lv3)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4783,7 +4763,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5108,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Special fan that was distributed at a big event.</t>
+          <t>Special fan that was distributed at a big event. (Air Turbulence Lv1)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5142,11 +5122,7 @@
           <t>Special fan that was distributed at a big event.</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5310,7 +5286,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>A gem with a power source within. Apparently created by fairies.</t>
+          <t>A self-powered gem. Apparently created by fairies. (Rainbow Flash Lv1)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5326,7 +5302,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -5531,7 +5507,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Spice that flows smoothly, which is good, because it must.</t>
+          <t>Spice that flows smoothly. Good, because it must. (Soul Absorb Lv3)</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5547,7 +5523,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6173,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Block of ice all too available in the distant northern seas.</t>
+          <t>Ice all too available in the distant northern seas. (Ice Edge Lv1)</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
@@ -6213,7 +6189,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -6235,7 +6211,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Unmeltable in fire of any temperature.</t>
+          <t>Unmeltable in fire of any temperature. (Ice Storm Lv1)</t>
         </is>
       </c>
       <c r="E162" t="inlineStr"/>
@@ -6249,11 +6225,7 @@
           <t>Unmeltable in fire of any temperature.</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6345,7 +6317,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Lets you stay one step ahead of the bad weather.</t>
+          <t>Lets you stay one step ahead of the bad weather. (Ice Storm Lv1)</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -6359,11 +6331,7 @@
           <t>Lets you stay one step ahead of the bad weather.</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -6451,7 +6419,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Red and white so you know it's auspicious. Only shaped like a turtle!</t>
+          <t>Auspicious red and white. Only turtle-shaped! (HP +100, 30% speed up)</t>
         </is>
       </c>
       <c r="E168" t="inlineStr"/>
@@ -6467,7 +6435,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -6523,7 +6491,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Spin it on its little stand and feel as if you rule the world.</t>
+          <t>Spin it and feel as if you rule the world. (Gaia Crush Lv2)</t>
         </is>
       </c>
       <c r="E170" t="inlineStr"/>
@@ -6539,7 +6507,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6529,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Made of a clear, shining crystal. It's missing one eye.</t>
+          <t>A clear, shining crystal. It's missing one eye. (Muon Plasma Lv1)</t>
         </is>
       </c>
       <c r="E171" t="inlineStr"/>
@@ -6577,7 +6545,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -7238,7 +7206,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>The seven-colored liquid that rainbows are made of.</t>
+          <t>The seven-colored liquid rainbows are made of. (Rainbow Flash Lv2)</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
@@ -7254,7 +7222,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -7485,7 +7453,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Drill, baby, drill! Pierce those heavens!</t>
+          <t>Drill, baby, drill! Pierce those heavens! (Stone Hammer Lv1)</t>
         </is>
       </c>
       <c r="E197" t="inlineStr"/>
@@ -7499,11 +7467,7 @@
           <t>Drill, baby, drill! Pierce those heavens!</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -7557,7 +7521,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Works on door-to-door salesmen and debt collectors.</t>
+          <t>Works on door-to-door salesmen and debt collectors. (enemies flee)</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -7571,11 +7535,7 @@
           <t>Works on door-to-door salesmen and debt collectors.</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -7595,7 +7555,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Fossil of some kind of interstellar cetacean.</t>
+          <t>Fossil of some kind of interstellar cetacean. (Soul Absorb Lv1)</t>
         </is>
       </c>
       <c r="E200" t="inlineStr"/>
@@ -7609,11 +7569,7 @@
           <t>Fossil of some kind of interstellar cetacean.</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -7633,7 +7589,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>The soil of a lost continent. Rich in potassium and mystery.</t>
+          <t>Lost continent soil. Rich in potassium and mystery. (Gaia Crush Lv2)</t>
         </is>
       </c>
       <c r="E201" t="inlineStr"/>
@@ -7649,7 +7605,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -7917,7 +7873,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Ancient doll so weird looking, it's gotta be extraterrestrial.</t>
+          <t>Ancient doll so weird, it's gotta be extraterrestrial. (Meteor Lv1)</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -7933,7 +7889,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -9516,7 +9472,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Burned when praying for rain. Works great... as prayers go.</t>
+          <t>Burned to pray for rain. Works great... as prayers go. (Ice Storm Lv2)</t>
         </is>
       </c>
       <c r="E254" t="inlineStr"/>
@@ -9532,7 +9488,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -9622,7 +9578,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Throw it and a violent tornado comes out.</t>
+          <t>Throw it and a violent tornado comes out. (Tempest Lv2)</t>
         </is>
       </c>
       <c r="E257" t="inlineStr"/>
@@ -9636,11 +9592,7 @@
           <t>Throw it and a violent tornado comes out.</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -10138,7 +10090,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Makes you feel somewhat quicker.</t>
+          <t>Makes you feel somewhat quicker. (25% speed up)</t>
         </is>
       </c>
       <c r="E271" t="inlineStr"/>
@@ -10152,11 +10104,7 @@
           <t>Makes you feel somewhat quicker (Speed +25%.).</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -10278,7 +10226,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Menorah that's smothered in blood. Definitely not kosher.</t>
+          <t>Menorah smothered in blood. Definitely not kosher. (Soul Absorb Lv5)</t>
         </is>
       </c>
       <c r="E275" t="inlineStr"/>
@@ -10294,7 +10242,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -10960,7 +10908,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Why let it expire it when you die? This license is forever.</t>
+          <t>Why let it expire when you die? Licensed forever. (40% speed up)</t>
         </is>
       </c>
       <c r="E294" t="inlineStr"/>
@@ -10976,7 +10924,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -10998,7 +10946,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Forgeries are more common than the genuine article.</t>
+          <t>Forgeries are more common than the genuine article. (60% speed up)</t>
         </is>
       </c>
       <c r="E295" t="inlineStr"/>
@@ -11012,11 +10960,7 @@
           <t>Forgeries are more common than the genuine article (Speed +60%.).</t>
         </is>
       </c>
-      <c r="H295" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -11036,7 +10980,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Raise your clock rate for a limited time.</t>
+          <t>Raise your clock rate for a while. (80% speed up, 60% evasion up)</t>
         </is>
       </c>
       <c r="E296" t="inlineStr"/>
@@ -11052,7 +10996,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -13758,7 +13702,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>The carbonation feels good as it slides down your throat.</t>
+          <t>The carbonation feels good sliding down your throat. (25% speed up)</t>
         </is>
       </c>
       <c r="E372" t="inlineStr"/>
@@ -13774,7 +13718,7 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -17619,7 +17563,7 @@
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>What you get when you toss a chunk of whale in your soup.</t>
+          <t>Toss whale in soup. Get this. (party HP +240, party cures freeze)</t>
         </is>
       </c>
       <c r="E478" t="inlineStr"/>
@@ -17635,7 +17579,7 @@
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(qol): what the program reading settled is shown
what the program reading settled is shown: Cover, Parry, four unique
skills, turns of summoned units, eight items
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_item_text.xlsx
+++ b/mod_project/data_tables/qol_item_text.xlsx
@@ -2145,7 +2145,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Those who join the Order receive this medal.</t>
+          <t>Those who join the Order receive this medal. (20% War Cry)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2155,11 +2155,7 @@
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2393,7 +2389,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>A fortunetelling book with a storied history.</t>
+          <t>A fortunetelling book with a storied history. (40% Accelerator)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2403,11 +2399,7 @@
         </is>
       </c>
       <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2777,7 +2769,7 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>no room for (50% sleep, 75% Accelerator): 89 characters</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5443,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Careful. Even though it's dead, it's still hungry.</t>
+          <t>Careful. Even though it's dead, it's still hungry. (lose 5% of gold)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
@@ -5461,11 +5453,7 @@
         </is>
       </c>
       <c r="G159" t="inlineStr"/>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5497,7 +5485,7 @@
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>no room for (lose 5% of gold): 81 characters</t>
         </is>
       </c>
     </row>
@@ -8083,7 +8071,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Burning ice that sleeps in the ocean's depths.</t>
+          <t>Burning ice that sleeps in the ocean's depths. (Fireball Lv3)</t>
         </is>
       </c>
       <c r="E243" t="inlineStr"/>
@@ -8093,11 +8081,7 @@
         </is>
       </c>
       <c r="G243" t="inlineStr"/>
-      <c r="H243" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -8151,7 +8135,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Emits a fell light and leads its owner to ruin.</t>
+          <t>Emits a fell light and leads its owner to ruin. (lose 5% of gold)</t>
         </is>
       </c>
       <c r="E245" t="inlineStr"/>
@@ -8161,11 +8145,7 @@
         </is>
       </c>
       <c r="G245" t="inlineStr"/>
-      <c r="H245" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -8245,7 +8225,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Apparently these are very expensive in some places.</t>
+          <t>Apparently these are very expensive in some places. (Fireball Lv3)</t>
         </is>
       </c>
       <c r="E248" t="inlineStr"/>
@@ -8255,11 +8235,7 @@
         </is>
       </c>
       <c r="G248" t="inlineStr"/>
-      <c r="H248" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -11135,7 +11111,7 @@
       <c r="G339" t="inlineStr"/>
       <c r="H339" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>no room for (HP/TP +360, 75% Accelerator): 78 characters</t>
         </is>
       </c>
     </row>
@@ -12239,7 +12215,7 @@
       <c r="G373" t="inlineStr"/>
       <c r="H373" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>no room for (25% Accelerator): 78 characters</t>
         </is>
       </c>
     </row>
@@ -12273,7 +12249,7 @@
       <c r="G374" t="inlineStr"/>
       <c r="H374" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>no room for (50% speed up, 50% Accelerator): 77 characters</t>
         </is>
       </c>
     </row>
@@ -13349,7 +13325,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>Potato chips covered with habanero powder.</t>
+          <t>Potato chips covered with habanero powder. (HP +120, 75% Accelerator)</t>
         </is>
       </c>
       <c r="E408" t="inlineStr"/>
@@ -13359,11 +13335,7 @@
         </is>
       </c>
       <c r="G408" t="inlineStr"/>
-      <c r="H408" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -13771,7 +13743,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Exquisite and jiggly almond-flavored tofu.</t>
+          <t>Exquisite and jiggly almond-flavored tofu. (TP +100, 50% Accelerator)</t>
         </is>
       </c>
       <c r="E421" t="inlineStr"/>
@@ -13781,11 +13753,7 @@
         </is>
       </c>
       <c r="G421" t="inlineStr"/>
-      <c r="H421" t="inlineStr">
-        <is>
-          <t>has an effect that is not decoded</t>
-        </is>
-      </c>
+      <c r="H421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">

</xml_diff>

<commit_message>
feat(qol): eleven more items, Demon Wall, Duration of the last dolls
eleven more items, Demon Wall, Duration of the last dolls, power of the
attacks of the player's summons
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_item_text.xlsx
+++ b/mod_project/data_tables/qol_item_text.xlsx
@@ -1561,7 +1561,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Beasts love it! The flavor and nutrition balance is just right.</t>
+          <t>Beasts love it! Flavor and nutrition just right. (30% HP to Beasts)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1573,7 +1573,7 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>A Souffle special. Goes off with a bang that makes you jump.</t>
+          <t>A Souffle special. Bang! (50% max HP damage up to 100, 75% stun)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -1675,7 +1675,7 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>A sedative for pregnant women, but there are side effects...</t>
+          <t>Pregnancy sedative. Side effects... (50% sleep, 75% Accelerator)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -2769,7 +2769,7 @@
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>no room for (50% sleep, 75% Accelerator): 89 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4597,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>An experimental pill created by a secret organization. Do not consume.</t>
+          <t>Secret organization pill. Do not eat. (50% max HP damage up to 100)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -4609,7 +4609,7 @@
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Liquor made of crushed fairies. Not guaranteed not to curse you...</t>
+          <t>Liquor of crushed fairies. (silences Apparitions, 25% petrifying)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -4771,7 +4771,7 @@
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -5473,7 +5473,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Piece of the stone under which there sleeps a king of gamblers.</t>
+          <t>Stone under which sleeps a king of gamblers. (lose 5% of gold)</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -5485,7 +5485,7 @@
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr">
         <is>
-          <t>no room for (lose 5% of gold): 81 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -8101,7 +8101,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Water with malicious intent. Good thing it's stuck in the bottle.</t>
+          <t>Malicious water, stuck in its bottle. (20% max HP damage up to 100)</t>
         </is>
       </c>
       <c r="E244" t="inlineStr"/>
@@ -8113,7 +8113,7 @@
       <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -8331,7 +8331,7 @@
       <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>no room for (15% max HP damage, 0.8% petrifying): 102 characters</t>
         </is>
       </c>
     </row>
@@ -11099,7 +11099,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Aged, well-smoked horse meat. An exquisite dish.</t>
+          <t>Aged, smoked horse meat. Exquisite. (HP/TP +360, 75% Accelerator)</t>
         </is>
       </c>
       <c r="E339" t="inlineStr"/>
@@ -11111,7 +11111,7 @@
       <c r="G339" t="inlineStr"/>
       <c r="H339" t="inlineStr">
         <is>
-          <t>no room for (HP/TP +360, 75% Accelerator): 78 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -11845,7 +11845,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>Food that smells like a public toilet that has gone uncleaned for years.</t>
+          <t>Smells like a filthy public toilet. (20% max HP damage up to 100)</t>
         </is>
       </c>
       <c r="E362" t="inlineStr"/>
@@ -11857,7 +11857,7 @@
       <c r="G362" t="inlineStr"/>
       <c r="H362" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -11879,7 +11879,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>So malodorous it's been mistaken for a chemical weapon.</t>
+          <t>Mistaken for a chemical weapon. (50% max HP damage up to 100)</t>
         </is>
       </c>
       <c r="E363" t="inlineStr"/>
@@ -11891,7 +11891,7 @@
       <c r="G363" t="inlineStr"/>
       <c r="H363" t="inlineStr">
         <is>
-          <t>has an effect that is not decoded</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -12203,7 +12203,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>It's sweet and spicy... What evil genius came up with this??</t>
+          <t>Sweet and spicy... What evil genius made this?? (25% Accelerator)</t>
         </is>
       </c>
       <c r="E373" t="inlineStr"/>
@@ -12215,7 +12215,7 @@
       <c r="G373" t="inlineStr"/>
       <c r="H373" t="inlineStr">
         <is>
-          <t>no room for (25% Accelerator): 78 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -12237,7 +12237,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>Hard to understand the point. Unbearably hot.</t>
+          <t>Pointless. Unbearably hot. (50% speed up, 50% Accelerator)</t>
         </is>
       </c>
       <c r="E374" t="inlineStr"/>
@@ -12249,7 +12249,7 @@
       <c r="G374" t="inlineStr"/>
       <c r="H374" t="inlineStr">
         <is>
-          <t>no room for (50% speed up, 50% Accelerator): 77 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
qol: apply joint skill TP/Pep costs
apply joint skill TP/Pep costs, expand doll pipe spacing, and refine
Dark Cloud text
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_item_text.xlsx
+++ b/mod_project/data_tables/qol_item_text.xlsx
@@ -4759,7 +4759,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Liquor of crushed fairies. (silences Apparitions, 25% petrifying)</t>
+          <t>Liquor of crushed fairies. (silences Apparitions, 25% petry)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Unfortunately, it's a one-way ticket. (10% petrifying)</t>
+          <t>Unfortunately, it's a one-way ticket. (10% petry)</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Honestly, just cut me some slack. (15% petrifying)</t>
+          <t>Honestly, just cut me some slack. (15% petry)</t>
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
@@ -8319,7 +8319,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>A roiling mass of darkness. And... is that a green lady in there?</t>
+          <t>Roiling mass. Is that a green lady in there? (15% HP dmg, 0.8% petry)</t>
         </is>
       </c>
       <c r="E251" t="inlineStr"/>
@@ -8331,7 +8331,7 @@
       <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr">
         <is>
-          <t>no room for (15% max HP damage, 0.8% petrifying): 102 characters</t>
+          <t>original sentence shortened to fit</t>
         </is>
       </c>
     </row>
@@ -9381,7 +9381,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>I really hope my photo's not on there. (15% petrifying)</t>
+          <t>I really hope my photo's not on there. (15% petry)</t>
         </is>
       </c>
       <c r="E284" t="inlineStr"/>

</xml_diff>